<commit_message>
finished full int-PID models and noise testing
</commit_message>
<xml_diff>
--- a/files/Controller Design/ZNMethods_ITAE_Errors.xlsx
+++ b/files/Controller Design/ZNMethods_ITAE_Errors.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulisboa-my.sharepoint.com/personal/ist1100262_tecnico_ulisboa_pt/Documents/MEMec/Thesis/files/Controller Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="170" documentId="8_{95F32091-D855-4402-ADD3-8991BE5FE270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{367E1D4A-7834-4649-B229-0E4FB1D0DB96}"/>
+  <xr:revisionPtr revIDLastSave="185" documentId="8_{95F32091-D855-4402-ADD3-8991BE5FE270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26216FB3-8594-41EA-B495-AA1D8894687A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" activeTab="1" xr2:uid="{6BCB78A0-0C46-4270-8084-079A19E30873}"/>
+    <workbookView xWindow="-3696" yWindow="-17388" windowWidth="30936" windowHeight="17496" activeTab="3" xr2:uid="{6BCB78A0-0C46-4270-8084-079A19E30873}"/>
   </bookViews>
   <sheets>
     <sheet name="CritGain" sheetId="1" r:id="rId1"/>
     <sheet name="PID_Models" sheetId="3" r:id="rId2"/>
     <sheet name="Gains" sheetId="5" r:id="rId3"/>
+    <sheet name="PID_Models_Noise" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="663">
   <si>
     <t>ν/ζ</t>
   </si>
@@ -2024,13 +2025,19 @@
   </si>
   <si>
     <t>1.5865</t>
+  </si>
+  <si>
+    <t>NOTE</t>
+  </si>
+  <si>
+    <t>Simulations kept over 30 seconds</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2054,6 +2061,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2456,7 +2470,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -2513,6 +2527,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2905,15 +2920,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07E4CF69-D65E-4E98-B411-A1D521930B25}">
   <dimension ref="B1:P43"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.90625" customWidth="1"/>
-    <col min="2" max="2" width="5.90625" customWidth="1"/>
-    <col min="3" max="12" width="7.6328125" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" customWidth="1"/>
+    <col min="2" max="2" width="5.88671875" customWidth="1"/>
+    <col min="3" max="12" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="33" t="s">
         <v>2</v>
       </c>
@@ -2921,7 +2936,7 @@
       <c r="D2" s="34"/>
       <c r="E2" s="35"/>
     </row>
-    <row r="3" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>9</v>
       </c>
@@ -2929,15 +2944,15 @@
       <c r="D3" s="31"/>
       <c r="E3" s="32"/>
     </row>
-    <row r="5" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="30" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="31"/>
       <c r="D6" s="32"/>
     </row>
-    <row r="7" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="20" t="s">
         <v>0</v>
       </c>
@@ -2978,7 +2993,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B8" s="13">
         <v>0.5</v>
       </c>
@@ -3020,7 +3035,7 @@
         <v>13.904676086956519</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="11">
         <v>0.7</v>
       </c>
@@ -3062,7 +3077,7 @@
         <v>2.8556499999999998</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10" s="11">
         <v>0.9</v>
       </c>
@@ -3104,7 +3119,7 @@
         <v>111.7454</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11" s="11">
         <v>1.1000000000000001</v>
       </c>
@@ -3146,7 +3161,7 @@
         <v>0.1535</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" s="11">
         <v>1.3</v>
       </c>
@@ -3183,7 +3198,7 @@
       <c r="M12" s="4"/>
       <c r="N12" s="5"/>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13" s="11">
         <v>1.5</v>
       </c>
@@ -3220,7 +3235,7 @@
       <c r="M13" s="4"/>
       <c r="N13" s="5"/>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="11">
         <v>1.7</v>
       </c>
@@ -3257,7 +3272,7 @@
       <c r="M14" s="4"/>
       <c r="N14" s="5"/>
     </row>
-    <row r="15" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="24">
         <v>1.9</v>
       </c>
@@ -3294,7 +3309,7 @@
       <c r="M15" s="6"/>
       <c r="N15" s="8"/>
     </row>
-    <row r="16" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="25" t="s">
         <v>11</v>
       </c>
@@ -3311,15 +3326,15 @@
       <c r="M16" s="26"/>
       <c r="N16" s="27"/>
     </row>
-    <row r="18" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="19" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="30" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="31"/>
       <c r="D19" s="32"/>
     </row>
-    <row r="20" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="20" t="s">
         <v>0</v>
       </c>
@@ -3360,7 +3375,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B21" s="13">
         <v>0.5</v>
       </c>
@@ -3402,7 +3417,7 @@
         <v>9.6706896551724139E-2</v>
       </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B22" s="11">
         <v>0.7</v>
       </c>
@@ -3444,7 +3459,7 @@
         <v>3.9E-2</v>
       </c>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B23" s="11">
         <v>0.9</v>
       </c>
@@ -3486,7 +3501,7 @@
         <v>0.65229999999999999</v>
       </c>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B24" s="11">
         <v>1.1000000000000001</v>
       </c>
@@ -3528,7 +3543,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B25" s="11">
         <v>1.3</v>
       </c>
@@ -3565,7 +3580,7 @@
       <c r="M25" s="4"/>
       <c r="N25" s="5"/>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B26" s="11">
         <v>1.5</v>
       </c>
@@ -3602,7 +3617,7 @@
       <c r="M26" s="4"/>
       <c r="N26" s="5"/>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B27" s="11">
         <v>1.7</v>
       </c>
@@ -3639,7 +3654,7 @@
       <c r="M27" s="4"/>
       <c r="N27" s="5"/>
     </row>
-    <row r="28" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="12">
         <v>1.9</v>
       </c>
@@ -3676,7 +3691,7 @@
       <c r="M28" s="6"/>
       <c r="N28" s="8"/>
     </row>
-    <row r="29" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="25" t="s">
         <v>12</v>
       </c>
@@ -3693,15 +3708,15 @@
       <c r="M29" s="26"/>
       <c r="N29" s="27"/>
     </row>
-    <row r="31" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="32" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="30" t="s">
         <v>15</v>
       </c>
       <c r="C32" s="31"/>
       <c r="D32" s="32"/>
     </row>
-    <row r="33" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="20" t="s">
         <v>0</v>
       </c>
@@ -3748,7 +3763,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B34" s="13">
         <v>0.5</v>
       </c>
@@ -3796,7 +3811,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B35" s="11">
         <v>0.7</v>
       </c>
@@ -3838,7 +3853,7 @@
         <v>0.10395</v>
       </c>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B36" s="11">
         <v>0.9</v>
       </c>
@@ -3880,7 +3895,7 @@
         <v>0.30299999999999999</v>
       </c>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B37" s="11">
         <v>1.1000000000000001</v>
       </c>
@@ -3922,7 +3937,7 @@
         <v>2.3999999999999998E-3</v>
       </c>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B38" s="11">
         <v>1.3</v>
       </c>
@@ -3959,7 +3974,7 @@
       <c r="M38" s="4"/>
       <c r="N38" s="5"/>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B39" s="11">
         <v>1.5</v>
       </c>
@@ -3996,7 +4011,7 @@
       <c r="M39" s="4"/>
       <c r="N39" s="5"/>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B40" s="11">
         <v>1.7</v>
       </c>
@@ -4033,7 +4048,7 @@
       <c r="M40" s="4"/>
       <c r="N40" s="5"/>
     </row>
-    <row r="41" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="12">
         <v>1.9</v>
       </c>
@@ -4070,7 +4085,7 @@
       <c r="M41" s="6"/>
       <c r="N41" s="8"/>
     </row>
-    <row r="42" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="25" t="s">
         <v>12</v>
       </c>
@@ -4087,7 +4102,7 @@
       <c r="M42" s="26"/>
       <c r="N42" s="27"/>
     </row>
-    <row r="43" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>25</v>
       </c>
@@ -4194,13 +4209,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6B8581E-0797-42DF-A936-58B89916A70A}">
   <dimension ref="B1:BP51"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="51" width="5.90625" customWidth="1"/>
+    <col min="3" max="51" width="5.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:68" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:68" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:68" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:68" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="20" t="s">
         <v>0</v>
       </c>
@@ -4397,7 +4412,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="3" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B3" s="1">
         <v>0.6</v>
       </c>
@@ -4594,7 +4609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B4" s="1">
         <v>0.7</v>
       </c>
@@ -4791,7 +4806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <v>0.8</v>
       </c>
@@ -4988,7 +5003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B6" s="1">
         <v>0.9</v>
       </c>
@@ -5185,7 +5200,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <v>1</v>
       </c>
@@ -5382,7 +5397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B8" s="1">
         <v>1.1000000000000001</v>
       </c>
@@ -5579,7 +5594,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <v>1.2</v>
       </c>
@@ -5776,7 +5791,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B10" s="1">
         <v>1.3</v>
       </c>
@@ -5973,7 +5988,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B11" s="1">
         <v>1.4</v>
       </c>
@@ -6170,7 +6185,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B12" s="1">
         <v>1.5</v>
       </c>
@@ -6367,7 +6382,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <v>1.6</v>
       </c>
@@ -6564,7 +6579,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B14" s="1">
         <v>1.7</v>
       </c>
@@ -6761,7 +6776,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B15" s="1">
         <v>1.8</v>
       </c>
@@ -6958,7 +6973,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B16" s="1">
         <v>1.9</v>
       </c>
@@ -7155,7 +7170,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:68" x14ac:dyDescent="0.3">
       <c r="BB17" s="1">
         <v>1.6</v>
       </c>
@@ -7202,7 +7217,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:68" x14ac:dyDescent="0.3">
       <c r="BB18" s="1">
         <v>1.7</v>
       </c>
@@ -7249,7 +7264,7 @@
         <v>18.8813</v>
       </c>
     </row>
-    <row r="19" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:68" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>24</v>
       </c>
@@ -7299,7 +7314,7 @@
         <v>16.979299999999999</v>
       </c>
     </row>
-    <row r="20" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:68" x14ac:dyDescent="0.3">
       <c r="BB20" s="1">
         <v>1.9</v>
       </c>
@@ -7346,7 +7361,7 @@
         <v>15.0428</v>
       </c>
     </row>
-    <row r="21" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:68" x14ac:dyDescent="0.3">
       <c r="BB21" s="1">
         <v>2</v>
       </c>
@@ -7393,7 +7408,7 @@
         <v>13.154400000000001</v>
       </c>
     </row>
-    <row r="22" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:68" x14ac:dyDescent="0.3">
       <c r="BB22" s="1">
         <v>2.1</v>
       </c>
@@ -7440,7 +7455,7 @@
         <v>11.366099999999999</v>
       </c>
     </row>
-    <row r="23" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:68" x14ac:dyDescent="0.3">
       <c r="BB23" s="1">
         <v>2.2000000000000002</v>
       </c>
@@ -7487,7 +7502,7 @@
         <v>9.7006999999999994</v>
       </c>
     </row>
-    <row r="24" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
         <v>283</v>
       </c>
@@ -7681,7 +7696,7 @@
         <v>8.1714000000000002</v>
       </c>
     </row>
-    <row r="25" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
         <v>304</v>
       </c>
@@ -7875,7 +7890,7 @@
         <v>6.7784000000000004</v>
       </c>
     </row>
-    <row r="26" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C26" t="s">
         <v>315</v>
       </c>
@@ -8069,7 +8084,7 @@
         <v>5.5202999999999998</v>
       </c>
     </row>
-    <row r="27" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
         <v>339</v>
       </c>
@@ -8263,7 +8278,7 @@
         <v>4.3936999999999999</v>
       </c>
     </row>
-    <row r="28" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C28" t="s">
         <v>354</v>
       </c>
@@ -8457,7 +8472,7 @@
         <v>3.3972000000000002</v>
       </c>
     </row>
-    <row r="29" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
         <v>360</v>
       </c>
@@ -8651,7 +8666,7 @@
         <v>2.5360999999999998</v>
       </c>
     </row>
-    <row r="30" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
         <v>389</v>
       </c>
@@ -8845,7 +8860,7 @@
         <v>1.8302</v>
       </c>
     </row>
-    <row r="31" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
         <v>10</v>
       </c>
@@ -9039,7 +9054,7 @@
         <v>1.3324</v>
       </c>
     </row>
-    <row r="32" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:68" x14ac:dyDescent="0.3">
       <c r="C32" t="s">
         <v>10</v>
       </c>
@@ -9233,7 +9248,7 @@
         <v>1.1324000000000001</v>
       </c>
     </row>
-    <row r="33" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="33" spans="3:68" x14ac:dyDescent="0.3">
       <c r="C33" t="s">
         <v>10</v>
       </c>
@@ -9427,7 +9442,7 @@
         <v>1.2544</v>
       </c>
     </row>
-    <row r="34" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="34" spans="3:68" x14ac:dyDescent="0.3">
       <c r="C34" t="s">
         <v>10</v>
       </c>
@@ -9621,7 +9636,7 @@
         <v>1.5032000000000001</v>
       </c>
     </row>
-    <row r="35" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="35" spans="3:68" x14ac:dyDescent="0.3">
       <c r="C35" t="s">
         <v>10</v>
       </c>
@@ -9815,7 +9830,7 @@
         <v>1.7546999999999999</v>
       </c>
     </row>
-    <row r="36" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="36" spans="3:68" x14ac:dyDescent="0.3">
       <c r="C36" t="s">
         <v>10</v>
       </c>
@@ -10009,7 +10024,7 @@
         <v>1.9636</v>
       </c>
     </row>
-    <row r="37" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="37" spans="3:68" x14ac:dyDescent="0.3">
       <c r="C37" t="s">
         <v>10</v>
       </c>
@@ -10203,7 +10218,7 @@
         <v>2.1153</v>
       </c>
     </row>
-    <row r="38" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="38" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB38" s="1">
         <v>3.7</v>
       </c>
@@ -10250,7 +10265,7 @@
         <v>2.2073999999999998</v>
       </c>
     </row>
-    <row r="39" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="39" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB39" s="1">
         <v>3.8</v>
       </c>
@@ -10297,7 +10312,7 @@
         <v>2.2433999999999998</v>
       </c>
     </row>
-    <row r="40" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="40" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB40" s="1">
         <v>3.9</v>
       </c>
@@ -10344,7 +10359,7 @@
         <v>2.2296</v>
       </c>
     </row>
-    <row r="41" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="41" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB41" s="1">
         <v>4</v>
       </c>
@@ -10391,7 +10406,7 @@
         <v>2.1762000000000001</v>
       </c>
     </row>
-    <row r="42" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="42" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB42" s="1">
         <v>4.0999999999999996</v>
       </c>
@@ -10438,7 +10453,7 @@
         <v>2.0937000000000001</v>
       </c>
     </row>
-    <row r="43" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="43" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB43" s="1">
         <v>4.2</v>
       </c>
@@ -10485,7 +10500,7 @@
         <v>1.9947999999999999</v>
       </c>
     </row>
-    <row r="44" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="44" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB44" s="1">
         <v>4.3</v>
       </c>
@@ -10532,7 +10547,7 @@
         <v>1.8925000000000001</v>
       </c>
     </row>
-    <row r="45" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="45" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB45" s="1">
         <v>4.4000000000000004</v>
       </c>
@@ -10579,7 +10594,7 @@
         <v>1.7986</v>
       </c>
     </row>
-    <row r="46" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="46" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB46" s="1">
         <v>4.5</v>
       </c>
@@ -10626,7 +10641,7 @@
         <v>1.7218</v>
       </c>
     </row>
-    <row r="47" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="47" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB47" s="1">
         <v>4.5999999999999996</v>
       </c>
@@ -10673,7 +10688,7 @@
         <v>1.6656</v>
       </c>
     </row>
-    <row r="48" spans="3:68" x14ac:dyDescent="0.35">
+    <row r="48" spans="3:68" x14ac:dyDescent="0.3">
       <c r="BB48" s="1">
         <v>4.7</v>
       </c>
@@ -10720,7 +10735,7 @@
         <v>1.6288</v>
       </c>
     </row>
-    <row r="49" spans="54:68" x14ac:dyDescent="0.35">
+    <row r="49" spans="54:68" x14ac:dyDescent="0.3">
       <c r="BB49" s="1">
         <v>4.8</v>
       </c>
@@ -10767,7 +10782,7 @@
         <v>1.6087</v>
       </c>
     </row>
-    <row r="50" spans="54:68" x14ac:dyDescent="0.35">
+    <row r="50" spans="54:68" x14ac:dyDescent="0.3">
       <c r="BB50" s="1">
         <v>4.9000000000000004</v>
       </c>
@@ -10814,7 +10829,7 @@
         <v>1.6042000000000001</v>
       </c>
     </row>
-    <row r="51" spans="54:68" x14ac:dyDescent="0.35">
+    <row r="51" spans="54:68" x14ac:dyDescent="0.3">
       <c r="BB51" s="1">
         <v>5</v>
       </c>
@@ -10894,32 +10909,32 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D68FACB-5B63-4831-A1B2-5F33785D9AB1}">
   <dimension ref="B2:AY81"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="51" width="6.26953125" customWidth="1"/>
+    <col min="3" max="51" width="6.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="7" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="9" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="2:51" ht="9" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="20" t="s">
         <v>0</v>
       </c>
@@ -11071,7 +11086,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B11" s="1">
         <v>0.6</v>
       </c>
@@ -11223,7 +11238,7 @@
         <v>48.9788</v>
       </c>
     </row>
-    <row r="12" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B12" s="1">
         <v>0.7</v>
       </c>
@@ -11375,7 +11390,7 @@
         <v>81.417500000000004</v>
       </c>
     </row>
-    <row r="13" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <v>0.8</v>
       </c>
@@ -11527,7 +11542,7 @@
         <v>92.267099999999999</v>
       </c>
     </row>
-    <row r="14" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B14" s="1">
         <v>0.9</v>
       </c>
@@ -11679,7 +11694,7 @@
         <v>81.819000000000003</v>
       </c>
     </row>
-    <row r="15" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B15" s="1">
         <v>1</v>
       </c>
@@ -11831,7 +11846,7 @@
         <v>63.426099999999998</v>
       </c>
     </row>
-    <row r="16" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B16" s="1">
         <v>1.1000000000000001</v>
       </c>
@@ -11983,7 +11998,7 @@
         <v>46.739899999999999</v>
       </c>
     </row>
-    <row r="17" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B17" s="1">
         <v>1.2</v>
       </c>
@@ -12135,7 +12150,7 @@
         <v>34.656199999999998</v>
       </c>
     </row>
-    <row r="18" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B18" s="1">
         <v>1.3</v>
       </c>
@@ -12287,7 +12302,7 @@
         <v>26.637</v>
       </c>
     </row>
-    <row r="19" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B19" s="1">
         <v>1.4</v>
       </c>
@@ -12439,7 +12454,7 @@
         <v>21.2818</v>
       </c>
     </row>
-    <row r="20" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B20" s="1">
         <v>1.5</v>
       </c>
@@ -12591,7 +12606,7 @@
         <v>17.2515</v>
       </c>
     </row>
-    <row r="21" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B21" s="1">
         <v>1.6</v>
       </c>
@@ -12743,7 +12758,7 @@
         <v>13.48</v>
       </c>
     </row>
-    <row r="22" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B22" s="1">
         <v>1.7</v>
       </c>
@@ -12895,7 +12910,7 @@
         <v>9.3887999999999998</v>
       </c>
     </row>
-    <row r="23" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B23" s="1">
         <v>1.8</v>
       </c>
@@ -13047,7 +13062,7 @@
         <v>5.2465999999999999</v>
       </c>
     </row>
-    <row r="24" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B24" s="1">
         <v>1.9</v>
       </c>
@@ -13199,15 +13214,15 @@
         <v>2.0608</v>
       </c>
     </row>
-    <row r="25" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="28" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="20" t="s">
         <v>0</v>
       </c>
@@ -13359,7 +13374,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B30" s="1">
         <v>0.6</v>
       </c>
@@ -13511,7 +13526,7 @@
         <v>4.6848999999999998</v>
       </c>
     </row>
-    <row r="31" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B31" s="1">
         <v>0.7</v>
       </c>
@@ -13663,7 +13678,7 @@
         <v>4.9732000000000003</v>
       </c>
     </row>
-    <row r="32" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B32" s="1">
         <v>0.8</v>
       </c>
@@ -13815,7 +13830,7 @@
         <v>5.3418999999999999</v>
       </c>
     </row>
-    <row r="33" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B33" s="1">
         <v>0.9</v>
       </c>
@@ -13967,7 +13982,7 @@
         <v>5.7504999999999997</v>
       </c>
     </row>
-    <row r="34" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B34" s="1">
         <v>1</v>
       </c>
@@ -14119,7 +14134,7 @@
         <v>6.1510999999999996</v>
       </c>
     </row>
-    <row r="35" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B35" s="1">
         <v>1.1000000000000001</v>
       </c>
@@ -14271,7 +14286,7 @@
         <v>6.4897999999999998</v>
       </c>
     </row>
-    <row r="36" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B36" s="1">
         <v>1.2</v>
       </c>
@@ -14423,7 +14438,7 @@
         <v>6.7114000000000003</v>
       </c>
     </row>
-    <row r="37" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B37" s="1">
         <v>1.3</v>
       </c>
@@ -14575,7 +14590,7 @@
         <v>6.7676999999999996</v>
       </c>
     </row>
-    <row r="38" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B38" s="1">
         <v>1.4</v>
       </c>
@@ -14727,7 +14742,7 @@
         <v>6.6273999999999997</v>
       </c>
     </row>
-    <row r="39" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B39" s="1">
         <v>1.5</v>
       </c>
@@ -14879,7 +14894,7 @@
         <v>6.2840999999999996</v>
       </c>
     </row>
-    <row r="40" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B40" s="1">
         <v>1.6</v>
       </c>
@@ -15031,7 +15046,7 @@
         <v>5.7587999999999999</v>
       </c>
     </row>
-    <row r="41" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B41" s="1">
         <v>1.7</v>
       </c>
@@ -15183,7 +15198,7 @@
         <v>5.0965999999999996</v>
       </c>
     </row>
-    <row r="42" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B42" s="1">
         <v>1.8</v>
       </c>
@@ -15335,7 +15350,7 @@
         <v>4.3577000000000004</v>
       </c>
     </row>
-    <row r="43" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B43" s="1">
         <v>1.9</v>
       </c>
@@ -15487,15 +15502,15 @@
         <v>3.6049000000000002</v>
       </c>
     </row>
-    <row r="44" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="45" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="46" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="47" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="20" t="s">
         <v>0</v>
       </c>
@@ -15647,7 +15662,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B49" s="1">
         <v>0.6</v>
       </c>
@@ -15799,7 +15814,7 @@
         <v>0.216</v>
       </c>
     </row>
-    <row r="50" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B50" s="1">
         <v>0.7</v>
       </c>
@@ -15951,7 +15966,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="51" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B51" s="1">
         <v>0.8</v>
       </c>
@@ -16103,7 +16118,7 @@
         <v>0.71130000000000004</v>
       </c>
     </row>
-    <row r="52" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B52" s="1">
         <v>0.9</v>
       </c>
@@ -16255,7 +16270,7 @@
         <v>2.1046999999999998</v>
       </c>
     </row>
-    <row r="53" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B53" s="1">
         <v>1</v>
       </c>
@@ -16407,7 +16422,7 @@
         <v>6.7112999999999996</v>
       </c>
     </row>
-    <row r="54" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B54" s="1">
         <v>1.1000000000000001</v>
       </c>
@@ -16559,7 +16574,7 @@
         <v>19.967700000000001</v>
       </c>
     </row>
-    <row r="55" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B55" s="1">
         <v>1.2</v>
       </c>
@@ -16711,7 +16726,7 @@
         <v>49.717100000000002</v>
       </c>
     </row>
-    <row r="56" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B56" s="1">
         <v>1.3</v>
       </c>
@@ -16863,7 +16878,7 @@
         <v>96.262900000000002</v>
       </c>
     </row>
-    <row r="57" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B57" s="1">
         <v>1.4</v>
       </c>
@@ -17015,7 +17030,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="58" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B58" s="1">
         <v>1.5</v>
       </c>
@@ -17167,7 +17182,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="59" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B59" s="1">
         <v>1.6</v>
       </c>
@@ -17319,7 +17334,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="60" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B60" s="1">
         <v>1.7</v>
       </c>
@@ -17471,7 +17486,7 @@
         <v>86.854799999999997</v>
       </c>
     </row>
-    <row r="61" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B61" s="1">
         <v>1.8</v>
       </c>
@@ -17623,7 +17638,7 @@
         <v>54.804000000000002</v>
       </c>
     </row>
-    <row r="62" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B62" s="1">
         <v>1.9</v>
       </c>
@@ -17775,15 +17790,15 @@
         <v>36.372300000000003</v>
       </c>
     </row>
-    <row r="63" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="64" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="65" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="66" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="65" spans="2:51" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="66" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B66" s="29" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B67" s="20" t="s">
         <v>0</v>
       </c>
@@ -17935,7 +17950,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B68" s="1">
         <v>0.6</v>
       </c>
@@ -18087,7 +18102,7 @@
         <v>122.8081</v>
       </c>
     </row>
-    <row r="69" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B69" s="1">
         <v>0.7</v>
       </c>
@@ -18239,7 +18254,7 @@
         <v>92.479100000000003</v>
       </c>
     </row>
-    <row r="70" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B70" s="1">
         <v>0.8</v>
       </c>
@@ -18391,7 +18406,7 @@
         <v>77.405799999999999</v>
       </c>
     </row>
-    <row r="71" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B71" s="1">
         <v>0.9</v>
       </c>
@@ -18543,7 +18558,7 @@
         <v>73.097499999999997</v>
       </c>
     </row>
-    <row r="72" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B72" s="1">
         <v>1</v>
       </c>
@@ -18695,7 +18710,7 @@
         <v>75.684700000000007</v>
       </c>
     </row>
-    <row r="73" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B73" s="1">
         <v>1.1000000000000001</v>
       </c>
@@ -18847,7 +18862,7 @@
         <v>81.919300000000007</v>
       </c>
     </row>
-    <row r="74" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B74" s="1">
         <v>1.2</v>
       </c>
@@ -18999,7 +19014,7 @@
         <v>89.174700000000001</v>
       </c>
     </row>
-    <row r="75" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B75" s="1">
         <v>1.3</v>
       </c>
@@ -19151,7 +19166,7 @@
         <v>95.445499999999996</v>
       </c>
     </row>
-    <row r="76" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B76" s="1">
         <v>1.4</v>
       </c>
@@ -19303,7 +19318,7 @@
         <v>99.347899999999996</v>
       </c>
     </row>
-    <row r="77" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B77" s="1">
         <v>1.5</v>
       </c>
@@ -19455,7 +19470,7 @@
         <v>100.1193</v>
       </c>
     </row>
-    <row r="78" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B78" s="1">
         <v>1.6</v>
       </c>
@@ -19607,7 +19622,7 @@
         <v>97.618499999999997</v>
       </c>
     </row>
-    <row r="79" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B79" s="1">
         <v>1.7</v>
       </c>
@@ -19759,7 +19774,7 @@
         <v>92.325900000000004</v>
       </c>
     </row>
-    <row r="80" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B80" s="1">
         <v>1.8</v>
       </c>
@@ -19911,7 +19926,7 @@
         <v>85.343000000000004</v>
       </c>
     </row>
-    <row r="81" spans="2:51" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:51" x14ac:dyDescent="0.3">
       <c r="B81" s="1">
         <v>1.9</v>
       </c>
@@ -20066,4 +20081,2318 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29424509-3824-4FC3-A99C-410B82A3A8E8}">
+  <dimension ref="B1:AY20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="51" width="6.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="K2" s="1">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M2" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="N2" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="O2" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="P2" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="R2" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="S2" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="T2" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="U2" s="1">
+        <v>2</v>
+      </c>
+      <c r="V2" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="W2" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="X2" s="1">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>2.4</v>
+      </c>
+      <c r="Z2" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="AA2" s="1">
+        <v>2.6</v>
+      </c>
+      <c r="AB2" s="1">
+        <v>2.7</v>
+      </c>
+      <c r="AC2" s="1">
+        <v>2.8</v>
+      </c>
+      <c r="AD2" s="1">
+        <v>2.9</v>
+      </c>
+      <c r="AE2" s="1">
+        <v>3</v>
+      </c>
+      <c r="AF2" s="1">
+        <v>3.1</v>
+      </c>
+      <c r="AG2" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="AH2" s="1">
+        <v>3.3</v>
+      </c>
+      <c r="AI2" s="1">
+        <v>3.4</v>
+      </c>
+      <c r="AJ2" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="AK2" s="1">
+        <v>3.6</v>
+      </c>
+      <c r="AL2" s="1">
+        <v>3.7</v>
+      </c>
+      <c r="AM2" s="1">
+        <v>3.8</v>
+      </c>
+      <c r="AN2" s="1">
+        <v>3.9</v>
+      </c>
+      <c r="AO2" s="1">
+        <v>4</v>
+      </c>
+      <c r="AP2" s="1">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AQ2" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="AR2" s="1">
+        <v>4.3</v>
+      </c>
+      <c r="AS2" s="1">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AT2" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="AU2" s="1">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AV2" s="1">
+        <v>4.7</v>
+      </c>
+      <c r="AW2" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="AX2" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="AY2" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B3" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="C3" s="1">
+        <v>7.0049999999999999</v>
+      </c>
+      <c r="D3" s="1">
+        <v>6.9410999999999996</v>
+      </c>
+      <c r="E3" s="1">
+        <v>6.8811</v>
+      </c>
+      <c r="F3" s="1">
+        <v>6.8255999999999997</v>
+      </c>
+      <c r="G3" s="1">
+        <v>6.7751000000000001</v>
+      </c>
+      <c r="H3" s="1">
+        <v>6.7259000000000002</v>
+      </c>
+      <c r="I3" s="1">
+        <v>6.673</v>
+      </c>
+      <c r="J3" s="1">
+        <v>6.6176000000000004</v>
+      </c>
+      <c r="K3" s="1">
+        <v>6.5576999999999996</v>
+      </c>
+      <c r="L3" s="1">
+        <v>6.49</v>
+      </c>
+      <c r="M3" s="1">
+        <v>6.4139999999999997</v>
+      </c>
+      <c r="N3" s="1">
+        <v>6.3312999999999997</v>
+      </c>
+      <c r="O3" s="1">
+        <v>6.2419000000000002</v>
+      </c>
+      <c r="P3" s="1">
+        <v>6.1445999999999996</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>6.0410000000000004</v>
+      </c>
+      <c r="R3" s="1">
+        <v>5.9336000000000002</v>
+      </c>
+      <c r="S3" s="1">
+        <v>5.8242000000000003</v>
+      </c>
+      <c r="T3" s="1">
+        <v>5.7130000000000001</v>
+      </c>
+      <c r="U3" s="1">
+        <v>5.6035000000000004</v>
+      </c>
+      <c r="V3" s="1">
+        <v>5.4987000000000004</v>
+      </c>
+      <c r="W3" s="1">
+        <v>5.3977000000000004</v>
+      </c>
+      <c r="X3" s="1">
+        <v>5.3037999999999998</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>5.2172999999999998</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>5.1360000000000001</v>
+      </c>
+      <c r="AA3" s="1">
+        <v>5.0602</v>
+      </c>
+      <c r="AB3" s="1">
+        <v>4.9874000000000001</v>
+      </c>
+      <c r="AC3" s="1">
+        <v>4.9223999999999997</v>
+      </c>
+      <c r="AD3" s="1">
+        <v>4.8632</v>
+      </c>
+      <c r="AE3" s="1">
+        <v>4.8102</v>
+      </c>
+      <c r="AF3" s="1">
+        <v>4.7584</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>4.7129000000000003</v>
+      </c>
+      <c r="AH3" s="1">
+        <v>4.6741999999999999</v>
+      </c>
+      <c r="AI3" s="1">
+        <v>4.6376999999999997</v>
+      </c>
+      <c r="AJ3" s="1">
+        <v>4.6052999999999997</v>
+      </c>
+      <c r="AK3" s="1">
+        <v>4.5789999999999997</v>
+      </c>
+      <c r="AL3" s="1">
+        <v>4.5557999999999996</v>
+      </c>
+      <c r="AM3" s="1">
+        <v>4.5376000000000003</v>
+      </c>
+      <c r="AN3" s="1">
+        <v>4.5248999999999997</v>
+      </c>
+      <c r="AO3" s="1">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="AP3" s="1">
+        <v>4.5267999999999997</v>
+      </c>
+      <c r="AQ3" s="1">
+        <v>4.5429000000000004</v>
+      </c>
+      <c r="AR3" s="1">
+        <v>4.5609999999999999</v>
+      </c>
+      <c r="AS3" s="1">
+        <v>4.5742000000000003</v>
+      </c>
+      <c r="AT3" s="1">
+        <v>4.5773000000000001</v>
+      </c>
+      <c r="AU3" s="1">
+        <v>4.5648</v>
+      </c>
+      <c r="AV3" s="1">
+        <v>4.5331000000000001</v>
+      </c>
+      <c r="AW3" s="1">
+        <v>4.4847999999999999</v>
+      </c>
+      <c r="AX3" s="1">
+        <v>4.4279000000000002</v>
+      </c>
+      <c r="AY3" s="1">
+        <v>4.3754999999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B4" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="C4" s="1">
+        <v>6.7342000000000004</v>
+      </c>
+      <c r="D4" s="1">
+        <v>6.6505999999999998</v>
+      </c>
+      <c r="E4" s="1">
+        <v>6.5789999999999997</v>
+      </c>
+      <c r="F4" s="1">
+        <v>6.5175000000000001</v>
+      </c>
+      <c r="G4" s="1">
+        <v>6.4650999999999996</v>
+      </c>
+      <c r="H4" s="1">
+        <v>6.4203000000000001</v>
+      </c>
+      <c r="I4" s="1">
+        <v>6.3788999999999998</v>
+      </c>
+      <c r="J4" s="1">
+        <v>6.3380000000000001</v>
+      </c>
+      <c r="K4" s="1">
+        <v>6.2950999999999997</v>
+      </c>
+      <c r="L4" s="1">
+        <v>6.2480000000000002</v>
+      </c>
+      <c r="M4" s="1">
+        <v>6.1954000000000002</v>
+      </c>
+      <c r="N4" s="1">
+        <v>6.1357999999999997</v>
+      </c>
+      <c r="O4" s="1">
+        <v>6.0701999999999998</v>
+      </c>
+      <c r="P4" s="1">
+        <v>5.9996</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>5.9252000000000002</v>
+      </c>
+      <c r="R4" s="1">
+        <v>5.8456000000000001</v>
+      </c>
+      <c r="S4" s="1">
+        <v>5.7614999999999998</v>
+      </c>
+      <c r="T4" s="1">
+        <v>5.6742999999999997</v>
+      </c>
+      <c r="U4" s="1">
+        <v>5.5853999999999999</v>
+      </c>
+      <c r="V4" s="1">
+        <v>5.4965000000000002</v>
+      </c>
+      <c r="W4" s="1">
+        <v>5.4089</v>
+      </c>
+      <c r="X4" s="1">
+        <v>5.3217999999999996</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>5.2370000000000001</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>5.1581999999999999</v>
+      </c>
+      <c r="AA4" s="1">
+        <v>5.0838999999999999</v>
+      </c>
+      <c r="AB4" s="1">
+        <v>5.0171999999999999</v>
+      </c>
+      <c r="AC4" s="1">
+        <v>4.9573</v>
+      </c>
+      <c r="AD4" s="1">
+        <v>4.9065000000000003</v>
+      </c>
+      <c r="AE4" s="1">
+        <v>4.8619000000000003</v>
+      </c>
+      <c r="AF4" s="1">
+        <v>4.8235999999999999</v>
+      </c>
+      <c r="AG4" s="1">
+        <v>4.7945000000000002</v>
+      </c>
+      <c r="AH4" s="1">
+        <v>4.7735000000000003</v>
+      </c>
+      <c r="AI4" s="1">
+        <v>4.7615999999999996</v>
+      </c>
+      <c r="AJ4" s="1">
+        <v>4.7576000000000001</v>
+      </c>
+      <c r="AK4" s="1">
+        <v>4.7610999999999999</v>
+      </c>
+      <c r="AL4" s="1">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="AM4" s="1">
+        <v>4.7850000000000001</v>
+      </c>
+      <c r="AN4" s="1">
+        <v>4.8076999999999996</v>
+      </c>
+      <c r="AO4" s="1">
+        <v>4.8335999999999997</v>
+      </c>
+      <c r="AP4" s="1">
+        <v>4.8582000000000001</v>
+      </c>
+      <c r="AQ4" s="1">
+        <v>4.8788999999999998</v>
+      </c>
+      <c r="AR4" s="1">
+        <v>4.8941999999999997</v>
+      </c>
+      <c r="AS4" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="AT4" s="1">
+        <v>4.8924000000000003</v>
+      </c>
+      <c r="AU4" s="1">
+        <v>4.8682999999999996</v>
+      </c>
+      <c r="AV4" s="1">
+        <v>4.8253000000000004</v>
+      </c>
+      <c r="AW4" s="1">
+        <v>4.7580999999999998</v>
+      </c>
+      <c r="AX4" s="1">
+        <v>4.6626000000000003</v>
+      </c>
+      <c r="AY4" s="1">
+        <v>4.5313999999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B5" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="C5" s="1">
+        <v>6.4707999999999997</v>
+      </c>
+      <c r="D5" s="1">
+        <v>6.3737000000000004</v>
+      </c>
+      <c r="E5" s="1">
+        <v>6.2859999999999996</v>
+      </c>
+      <c r="F5" s="1">
+        <v>6.2130999999999998</v>
+      </c>
+      <c r="G5" s="1">
+        <v>6.1551</v>
+      </c>
+      <c r="H5" s="1">
+        <v>6.1085000000000003</v>
+      </c>
+      <c r="I5" s="1">
+        <v>6.0694999999999997</v>
+      </c>
+      <c r="J5" s="1">
+        <v>6.0353000000000003</v>
+      </c>
+      <c r="K5" s="1">
+        <v>6.0050999999999997</v>
+      </c>
+      <c r="L5" s="1">
+        <v>5.9774000000000003</v>
+      </c>
+      <c r="M5" s="1">
+        <v>5.9470000000000001</v>
+      </c>
+      <c r="N5" s="1">
+        <v>5.9130000000000003</v>
+      </c>
+      <c r="O5" s="1">
+        <v>5.8738000000000001</v>
+      </c>
+      <c r="P5" s="1">
+        <v>5.8291000000000004</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>5.7797999999999998</v>
+      </c>
+      <c r="R5" s="1">
+        <v>5.7256</v>
+      </c>
+      <c r="S5" s="1">
+        <v>5.6670999999999996</v>
+      </c>
+      <c r="T5" s="1">
+        <v>5.6059000000000001</v>
+      </c>
+      <c r="U5" s="1">
+        <v>5.5423999999999998</v>
+      </c>
+      <c r="V5" s="1">
+        <v>5.4771999999999998</v>
+      </c>
+      <c r="W5" s="1">
+        <v>5.4109999999999996</v>
+      </c>
+      <c r="X5" s="1">
+        <v>5.3461999999999996</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>5.2835000000000001</v>
+      </c>
+      <c r="Z5" s="1">
+        <v>5.2224000000000004</v>
+      </c>
+      <c r="AA5" s="1">
+        <v>5.1646999999999998</v>
+      </c>
+      <c r="AB5" s="1">
+        <v>5.1124999999999998</v>
+      </c>
+      <c r="AC5" s="1">
+        <v>5.0643000000000002</v>
+      </c>
+      <c r="AD5" s="1">
+        <v>5.0217999999999998</v>
+      </c>
+      <c r="AE5" s="1">
+        <v>4.9858000000000002</v>
+      </c>
+      <c r="AF5" s="1">
+        <v>4.9553000000000003</v>
+      </c>
+      <c r="AG5" s="1">
+        <v>4.9314</v>
+      </c>
+      <c r="AH5" s="1">
+        <v>4.9127000000000001</v>
+      </c>
+      <c r="AI5" s="1">
+        <v>4.8998999999999997</v>
+      </c>
+      <c r="AJ5" s="1">
+        <v>4.8928000000000003</v>
+      </c>
+      <c r="AK5" s="1">
+        <v>4.8903999999999996</v>
+      </c>
+      <c r="AL5" s="1">
+        <v>4.8921999999999999</v>
+      </c>
+      <c r="AM5" s="1">
+        <v>4.8979999999999997</v>
+      </c>
+      <c r="AN5" s="1">
+        <v>4.9058000000000002</v>
+      </c>
+      <c r="AO5" s="1">
+        <v>4.9141000000000004</v>
+      </c>
+      <c r="AP5" s="1">
+        <v>4.9227999999999996</v>
+      </c>
+      <c r="AQ5" s="1">
+        <v>4.9275000000000002</v>
+      </c>
+      <c r="AR5" s="1">
+        <v>4.9259000000000004</v>
+      </c>
+      <c r="AS5" s="1">
+        <v>4.9147999999999996</v>
+      </c>
+      <c r="AT5" s="1">
+        <v>4.8905000000000003</v>
+      </c>
+      <c r="AU5" s="1">
+        <v>4.8513999999999999</v>
+      </c>
+      <c r="AV5" s="1">
+        <v>4.7927999999999997</v>
+      </c>
+      <c r="AW5" s="1">
+        <v>4.7089999999999996</v>
+      </c>
+      <c r="AX5" s="1">
+        <v>4.5964</v>
+      </c>
+      <c r="AY5" s="1">
+        <v>4.4503000000000004</v>
+      </c>
+    </row>
+    <row r="6" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B6" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="C6" s="1">
+        <v>6.1817000000000002</v>
+      </c>
+      <c r="D6" s="1">
+        <v>6.0883000000000003</v>
+      </c>
+      <c r="E6" s="1">
+        <v>5.9993999999999996</v>
+      </c>
+      <c r="F6" s="1">
+        <v>5.9195000000000002</v>
+      </c>
+      <c r="G6" s="1">
+        <v>5.8539000000000003</v>
+      </c>
+      <c r="H6" s="1">
+        <v>5.8041999999999998</v>
+      </c>
+      <c r="I6" s="1">
+        <v>5.7672999999999996</v>
+      </c>
+      <c r="J6" s="1">
+        <v>5.7397999999999998</v>
+      </c>
+      <c r="K6" s="1">
+        <v>5.718</v>
+      </c>
+      <c r="L6" s="1">
+        <v>5.6989000000000001</v>
+      </c>
+      <c r="M6" s="1">
+        <v>5.6805000000000003</v>
+      </c>
+      <c r="N6" s="1">
+        <v>5.6616</v>
+      </c>
+      <c r="O6" s="1">
+        <v>5.6405000000000003</v>
+      </c>
+      <c r="P6" s="1">
+        <v>5.6158999999999999</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>5.5875000000000004</v>
+      </c>
+      <c r="R6" s="1">
+        <v>5.5553999999999997</v>
+      </c>
+      <c r="S6" s="1">
+        <v>5.5198</v>
+      </c>
+      <c r="T6" s="1">
+        <v>5.4809999999999999</v>
+      </c>
+      <c r="U6" s="1">
+        <v>5.4397000000000002</v>
+      </c>
+      <c r="V6" s="1">
+        <v>5.3963999999999999</v>
+      </c>
+      <c r="W6" s="1">
+        <v>5.3521000000000001</v>
+      </c>
+      <c r="X6" s="1">
+        <v>5.3078000000000003</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>5.2630999999999997</v>
+      </c>
+      <c r="Z6" s="1">
+        <v>5.2180999999999997</v>
+      </c>
+      <c r="AA6" s="1">
+        <v>5.1734999999999998</v>
+      </c>
+      <c r="AB6" s="1">
+        <v>5.1295000000000002</v>
+      </c>
+      <c r="AC6" s="1">
+        <v>5.0872999999999999</v>
+      </c>
+      <c r="AD6" s="1">
+        <v>5.0483000000000002</v>
+      </c>
+      <c r="AE6" s="1">
+        <v>5.0114000000000001</v>
+      </c>
+      <c r="AF6" s="1">
+        <v>4.9771999999999998</v>
+      </c>
+      <c r="AG6" s="1">
+        <v>4.9477000000000002</v>
+      </c>
+      <c r="AH6" s="1">
+        <v>4.9222000000000001</v>
+      </c>
+      <c r="AI6" s="1">
+        <v>4.9001999999999999</v>
+      </c>
+      <c r="AJ6" s="1">
+        <v>4.8807999999999998</v>
+      </c>
+      <c r="AK6" s="1">
+        <v>4.8646000000000003</v>
+      </c>
+      <c r="AL6" s="1">
+        <v>4.8506999999999998</v>
+      </c>
+      <c r="AM6" s="1">
+        <v>4.8376999999999999</v>
+      </c>
+      <c r="AN6" s="1">
+        <v>4.8251999999999997</v>
+      </c>
+      <c r="AO6" s="1">
+        <v>4.8120000000000003</v>
+      </c>
+      <c r="AP6" s="1">
+        <v>4.8010999999999999</v>
+      </c>
+      <c r="AQ6" s="1">
+        <v>4.7869000000000002</v>
+      </c>
+      <c r="AR6" s="1">
+        <v>4.7656999999999998</v>
+      </c>
+      <c r="AS6" s="1">
+        <v>4.7343000000000002</v>
+      </c>
+      <c r="AT6" s="1">
+        <v>4.6902999999999997</v>
+      </c>
+      <c r="AU6" s="1">
+        <v>4.6334999999999997</v>
+      </c>
+      <c r="AV6" s="1">
+        <v>4.5559000000000003</v>
+      </c>
+      <c r="AW6" s="1">
+        <v>4.4527000000000001</v>
+      </c>
+      <c r="AX6" s="1">
+        <v>4.3193999999999999</v>
+      </c>
+      <c r="AY6" s="1">
+        <v>4.1529999999999996</v>
+      </c>
+    </row>
+    <row r="7" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1">
+        <v>5.7971000000000004</v>
+      </c>
+      <c r="D7" s="1">
+        <v>5.7145999999999999</v>
+      </c>
+      <c r="E7" s="1">
+        <v>5.6444999999999999</v>
+      </c>
+      <c r="F7" s="1">
+        <v>5.5877999999999997</v>
+      </c>
+      <c r="G7" s="1">
+        <v>5.5431999999999997</v>
+      </c>
+      <c r="H7" s="1">
+        <v>5.5044000000000004</v>
+      </c>
+      <c r="I7" s="1">
+        <v>5.4739000000000004</v>
+      </c>
+      <c r="J7" s="1">
+        <v>5.4550000000000001</v>
+      </c>
+      <c r="K7" s="1">
+        <v>5.4451000000000001</v>
+      </c>
+      <c r="L7" s="1">
+        <v>5.4408000000000003</v>
+      </c>
+      <c r="M7" s="1">
+        <v>5.4386000000000001</v>
+      </c>
+      <c r="N7" s="1">
+        <v>5.4367000000000001</v>
+      </c>
+      <c r="O7" s="1">
+        <v>5.4337999999999997</v>
+      </c>
+      <c r="P7" s="1">
+        <v>5.4291999999999998</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>5.4222999999999999</v>
+      </c>
+      <c r="R7" s="1">
+        <v>5.4127999999999998</v>
+      </c>
+      <c r="S7" s="1">
+        <v>5.4008000000000003</v>
+      </c>
+      <c r="T7" s="1">
+        <v>5.3861999999999997</v>
+      </c>
+      <c r="U7" s="1">
+        <v>5.3695000000000004</v>
+      </c>
+      <c r="V7" s="1">
+        <v>5.3506999999999998</v>
+      </c>
+      <c r="W7" s="1">
+        <v>5.3303000000000003</v>
+      </c>
+      <c r="X7" s="1">
+        <v>5.3085000000000004</v>
+      </c>
+      <c r="Y7" s="1">
+        <v>5.2853000000000003</v>
+      </c>
+      <c r="Z7" s="1">
+        <v>5.2607999999999997</v>
+      </c>
+      <c r="AA7" s="1">
+        <v>5.2351000000000001</v>
+      </c>
+      <c r="AB7" s="1">
+        <v>5.2081</v>
+      </c>
+      <c r="AC7" s="1">
+        <v>5.1802000000000001</v>
+      </c>
+      <c r="AD7" s="1">
+        <v>5.1512000000000002</v>
+      </c>
+      <c r="AE7" s="1">
+        <v>5.1208</v>
+      </c>
+      <c r="AF7" s="1">
+        <v>5.0892999999999997</v>
+      </c>
+      <c r="AG7" s="1">
+        <v>5.0567000000000002</v>
+      </c>
+      <c r="AH7" s="1">
+        <v>5.0229999999999997</v>
+      </c>
+      <c r="AI7" s="1">
+        <v>4.9881000000000002</v>
+      </c>
+      <c r="AJ7" s="1">
+        <v>4.9523000000000001</v>
+      </c>
+      <c r="AK7" s="1">
+        <v>4.9168000000000003</v>
+      </c>
+      <c r="AL7" s="1">
+        <v>4.8817000000000004</v>
+      </c>
+      <c r="AM7" s="1">
+        <v>4.8460999999999999</v>
+      </c>
+      <c r="AN7" s="1">
+        <v>4.8076999999999996</v>
+      </c>
+      <c r="AO7" s="1">
+        <v>4.7676999999999996</v>
+      </c>
+      <c r="AP7" s="1">
+        <v>4.7237</v>
+      </c>
+      <c r="AQ7" s="1">
+        <v>4.6741999999999999</v>
+      </c>
+      <c r="AR7" s="1">
+        <v>4.6214000000000004</v>
+      </c>
+      <c r="AS7" s="1">
+        <v>4.5654000000000003</v>
+      </c>
+      <c r="AT7" s="1">
+        <v>4.4988000000000001</v>
+      </c>
+      <c r="AU7" s="1">
+        <v>4.4192</v>
+      </c>
+      <c r="AV7" s="1">
+        <v>4.3177000000000003</v>
+      </c>
+      <c r="AW7" s="1">
+        <v>4.1917</v>
+      </c>
+      <c r="AX7" s="1">
+        <v>4.0472000000000001</v>
+      </c>
+      <c r="AY7" s="1">
+        <v>3.8944999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B8" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C8" s="1">
+        <v>5.1003999999999996</v>
+      </c>
+      <c r="D8" s="1">
+        <v>5.1925999999999997</v>
+      </c>
+      <c r="E8" s="1">
+        <v>5.2519999999999998</v>
+      </c>
+      <c r="F8" s="1">
+        <v>5.2332000000000001</v>
+      </c>
+      <c r="G8" s="1">
+        <v>5.19</v>
+      </c>
+      <c r="H8" s="1">
+        <v>5.1543000000000001</v>
+      </c>
+      <c r="I8" s="1">
+        <v>5.1253000000000002</v>
+      </c>
+      <c r="J8" s="1">
+        <v>5.1146000000000003</v>
+      </c>
+      <c r="K8" s="1">
+        <v>5.1196999999999999</v>
+      </c>
+      <c r="L8" s="1">
+        <v>5.1349</v>
+      </c>
+      <c r="M8" s="1">
+        <v>5.1546000000000003</v>
+      </c>
+      <c r="N8" s="1">
+        <v>5.1775000000000002</v>
+      </c>
+      <c r="O8" s="1">
+        <v>5.2007000000000003</v>
+      </c>
+      <c r="P8" s="1">
+        <v>5.2225999999999999</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>5.2431000000000001</v>
+      </c>
+      <c r="R8" s="1">
+        <v>5.2609000000000004</v>
+      </c>
+      <c r="S8" s="1">
+        <v>5.2763</v>
+      </c>
+      <c r="T8" s="1">
+        <v>5.2910000000000004</v>
+      </c>
+      <c r="U8" s="1">
+        <v>5.3029999999999999</v>
+      </c>
+      <c r="V8" s="1">
+        <v>5.3128000000000002</v>
+      </c>
+      <c r="W8" s="1">
+        <v>5.3205999999999998</v>
+      </c>
+      <c r="X8" s="1">
+        <v>5.3262</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>5.33</v>
+      </c>
+      <c r="Z8" s="1">
+        <v>5.3315999999999999</v>
+      </c>
+      <c r="AA8" s="1">
+        <v>5.3311999999999999</v>
+      </c>
+      <c r="AB8" s="1">
+        <v>5.3288000000000002</v>
+      </c>
+      <c r="AC8" s="1">
+        <v>5.3242000000000003</v>
+      </c>
+      <c r="AD8" s="1">
+        <v>5.3174000000000001</v>
+      </c>
+      <c r="AE8" s="1">
+        <v>5.3080999999999996</v>
+      </c>
+      <c r="AF8" s="1">
+        <v>5.2961999999999998</v>
+      </c>
+      <c r="AG8" s="1">
+        <v>5.2816000000000001</v>
+      </c>
+      <c r="AH8" s="1">
+        <v>5.2640000000000002</v>
+      </c>
+      <c r="AI8" s="1">
+        <v>5.2431999999999999</v>
+      </c>
+      <c r="AJ8" s="1">
+        <v>5.2194000000000003</v>
+      </c>
+      <c r="AK8" s="1">
+        <v>5.1923000000000004</v>
+      </c>
+      <c r="AL8" s="1">
+        <v>5.1614000000000004</v>
+      </c>
+      <c r="AM8" s="1">
+        <v>5.1261000000000001</v>
+      </c>
+      <c r="AN8" s="1">
+        <v>5.0872000000000002</v>
+      </c>
+      <c r="AO8" s="1">
+        <v>5.0435999999999996</v>
+      </c>
+      <c r="AP8" s="1">
+        <v>4.9935</v>
+      </c>
+      <c r="AQ8" s="1">
+        <v>4.9375999999999998</v>
+      </c>
+      <c r="AR8" s="1">
+        <v>4.8734000000000002</v>
+      </c>
+      <c r="AS8" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="AT8" s="1">
+        <v>4.7153</v>
+      </c>
+      <c r="AU8" s="1">
+        <v>4.6193999999999997</v>
+      </c>
+      <c r="AV8" s="1">
+        <v>4.5124000000000004</v>
+      </c>
+      <c r="AW8" s="1">
+        <v>4.3978999999999999</v>
+      </c>
+      <c r="AX8" s="1">
+        <v>4.2811000000000003</v>
+      </c>
+      <c r="AY8" s="1">
+        <v>4.1715</v>
+      </c>
+    </row>
+    <row r="9" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B9" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="C9" s="1">
+        <v>5.2290000000000001</v>
+      </c>
+      <c r="D9" s="1">
+        <v>5.2933000000000003</v>
+      </c>
+      <c r="E9" s="1">
+        <v>5.1527000000000003</v>
+      </c>
+      <c r="F9" s="1">
+        <v>4.9878</v>
+      </c>
+      <c r="G9" s="1">
+        <v>4.8154000000000003</v>
+      </c>
+      <c r="H9" s="1">
+        <v>4.7541000000000002</v>
+      </c>
+      <c r="I9" s="1">
+        <v>4.7270000000000003</v>
+      </c>
+      <c r="J9" s="1">
+        <v>4.7089999999999996</v>
+      </c>
+      <c r="K9" s="1">
+        <v>4.7178000000000004</v>
+      </c>
+      <c r="L9" s="1">
+        <v>4.7398999999999996</v>
+      </c>
+      <c r="M9" s="1">
+        <v>4.7835000000000001</v>
+      </c>
+      <c r="N9" s="1">
+        <v>4.8327999999999998</v>
+      </c>
+      <c r="O9" s="1">
+        <v>4.8826999999999998</v>
+      </c>
+      <c r="P9" s="1">
+        <v>4.9313000000000002</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>4.9778000000000002</v>
+      </c>
+      <c r="R9" s="1">
+        <v>5.0209000000000001</v>
+      </c>
+      <c r="S9" s="1">
+        <v>5.0599999999999996</v>
+      </c>
+      <c r="T9" s="1">
+        <v>5.0971000000000002</v>
+      </c>
+      <c r="U9" s="1">
+        <v>5.1330999999999998</v>
+      </c>
+      <c r="V9" s="1">
+        <v>5.1681999999999997</v>
+      </c>
+      <c r="W9" s="1">
+        <v>5.2019000000000002</v>
+      </c>
+      <c r="X9" s="1">
+        <v>5.2348999999999997</v>
+      </c>
+      <c r="Y9" s="1">
+        <v>5.266</v>
+      </c>
+      <c r="Z9" s="1">
+        <v>5.2965999999999998</v>
+      </c>
+      <c r="AA9" s="1">
+        <v>5.3250999999999999</v>
+      </c>
+      <c r="AB9" s="1">
+        <v>5.3506999999999998</v>
+      </c>
+      <c r="AC9" s="1">
+        <v>5.3731</v>
+      </c>
+      <c r="AD9" s="1">
+        <v>5.3925999999999998</v>
+      </c>
+      <c r="AE9" s="1">
+        <v>5.4089999999999998</v>
+      </c>
+      <c r="AF9" s="1">
+        <v>5.4226999999999999</v>
+      </c>
+      <c r="AG9" s="1">
+        <v>5.4337</v>
+      </c>
+      <c r="AH9" s="1">
+        <v>5.4414999999999996</v>
+      </c>
+      <c r="AI9" s="1">
+        <v>5.4459</v>
+      </c>
+      <c r="AJ9" s="1">
+        <v>5.4473000000000003</v>
+      </c>
+      <c r="AK9" s="1">
+        <v>5.4452999999999996</v>
+      </c>
+      <c r="AL9" s="1">
+        <v>5.4398</v>
+      </c>
+      <c r="AM9" s="1">
+        <v>5.4307999999999996</v>
+      </c>
+      <c r="AN9" s="1">
+        <v>5.4179000000000004</v>
+      </c>
+      <c r="AO9" s="1">
+        <v>5.4013999999999998</v>
+      </c>
+      <c r="AP9" s="1">
+        <v>5.3807</v>
+      </c>
+      <c r="AQ9" s="1">
+        <v>5.3552999999999997</v>
+      </c>
+      <c r="AR9" s="1">
+        <v>5.3246000000000002</v>
+      </c>
+      <c r="AS9" s="1">
+        <v>5.2885</v>
+      </c>
+      <c r="AT9" s="1">
+        <v>5.2468000000000004</v>
+      </c>
+      <c r="AU9" s="1">
+        <v>5.2011000000000003</v>
+      </c>
+      <c r="AV9" s="1">
+        <v>5.1513</v>
+      </c>
+      <c r="AW9" s="1">
+        <v>5.1001000000000003</v>
+      </c>
+      <c r="AX9" s="1">
+        <v>5.0537999999999998</v>
+      </c>
+      <c r="AY9" s="1">
+        <v>5.0296000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B10" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1">
+        <v>5.5411000000000001</v>
+      </c>
+      <c r="E10" s="1">
+        <v>5.0861000000000001</v>
+      </c>
+      <c r="F10" s="1">
+        <v>4.8479999999999999</v>
+      </c>
+      <c r="G10" s="1">
+        <v>4.6717000000000004</v>
+      </c>
+      <c r="H10" s="1">
+        <v>4.4744999999999999</v>
+      </c>
+      <c r="I10" s="1">
+        <v>4.3411</v>
+      </c>
+      <c r="J10" s="1">
+        <v>4.2411000000000003</v>
+      </c>
+      <c r="K10" s="1">
+        <v>4.2054999999999998</v>
+      </c>
+      <c r="L10" s="1">
+        <v>4.2323000000000004</v>
+      </c>
+      <c r="M10" s="1">
+        <v>4.2927</v>
+      </c>
+      <c r="N10" s="1">
+        <v>4.3624000000000001</v>
+      </c>
+      <c r="O10" s="1">
+        <v>4.4328000000000003</v>
+      </c>
+      <c r="P10" s="1">
+        <v>4.5026000000000002</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>4.5709999999999997</v>
+      </c>
+      <c r="R10" s="1">
+        <v>4.6375999999999999</v>
+      </c>
+      <c r="S10" s="1">
+        <v>4.6996000000000002</v>
+      </c>
+      <c r="T10" s="1">
+        <v>4.7615999999999996</v>
+      </c>
+      <c r="U10" s="1">
+        <v>4.8231000000000002</v>
+      </c>
+      <c r="V10" s="1">
+        <v>4.8783000000000003</v>
+      </c>
+      <c r="W10" s="1">
+        <v>4.9336000000000002</v>
+      </c>
+      <c r="X10" s="1">
+        <v>4.9866999999999999</v>
+      </c>
+      <c r="Y10" s="1">
+        <v>5.0374999999999996</v>
+      </c>
+      <c r="Z10" s="1">
+        <v>5.0850999999999997</v>
+      </c>
+      <c r="AA10" s="1">
+        <v>5.1311</v>
+      </c>
+      <c r="AB10" s="1">
+        <v>5.1759000000000004</v>
+      </c>
+      <c r="AC10" s="1">
+        <v>5.2198000000000002</v>
+      </c>
+      <c r="AD10" s="1">
+        <v>5.2630999999999997</v>
+      </c>
+      <c r="AE10" s="1">
+        <v>5.3045999999999998</v>
+      </c>
+      <c r="AF10" s="1">
+        <v>5.3448000000000002</v>
+      </c>
+      <c r="AG10" s="1">
+        <v>5.3826000000000001</v>
+      </c>
+      <c r="AH10" s="1">
+        <v>5.4170999999999996</v>
+      </c>
+      <c r="AI10" s="1">
+        <v>5.4477000000000002</v>
+      </c>
+      <c r="AJ10" s="1">
+        <v>5.4751000000000003</v>
+      </c>
+      <c r="AK10" s="1">
+        <v>5.4988999999999999</v>
+      </c>
+      <c r="AL10" s="1">
+        <v>5.5197000000000003</v>
+      </c>
+      <c r="AM10" s="1">
+        <v>5.5377999999999998</v>
+      </c>
+      <c r="AN10" s="1">
+        <v>5.5532000000000004</v>
+      </c>
+      <c r="AO10" s="1">
+        <v>5.5659999999999998</v>
+      </c>
+      <c r="AP10" s="1">
+        <v>5.5762999999999998</v>
+      </c>
+      <c r="AQ10" s="1">
+        <v>5.5845000000000002</v>
+      </c>
+      <c r="AR10" s="1">
+        <v>5.5911999999999997</v>
+      </c>
+      <c r="AS10" s="1">
+        <v>5.5963000000000003</v>
+      </c>
+      <c r="AT10" s="1">
+        <v>5.6003999999999996</v>
+      </c>
+      <c r="AU10" s="1">
+        <v>5.6067999999999998</v>
+      </c>
+      <c r="AV10" s="1">
+        <v>5.6181999999999999</v>
+      </c>
+      <c r="AW10" s="1">
+        <v>5.6394000000000002</v>
+      </c>
+      <c r="AX10" s="1">
+        <v>5.6792999999999996</v>
+      </c>
+      <c r="AY10" s="1">
+        <v>5.7618999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B11" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="1">
+        <v>5.6300999999999997</v>
+      </c>
+      <c r="F11" s="1">
+        <v>5.0602999999999998</v>
+      </c>
+      <c r="G11" s="1">
+        <v>4.7470999999999997</v>
+      </c>
+      <c r="H11" s="1">
+        <v>4.4408000000000003</v>
+      </c>
+      <c r="I11" s="1">
+        <v>4.1014999999999997</v>
+      </c>
+      <c r="J11" s="1">
+        <v>3.8090999999999999</v>
+      </c>
+      <c r="K11" s="1">
+        <v>3.6943000000000001</v>
+      </c>
+      <c r="L11" s="1">
+        <v>3.7033999999999998</v>
+      </c>
+      <c r="M11" s="1">
+        <v>3.7475000000000001</v>
+      </c>
+      <c r="N11" s="1">
+        <v>3.8107000000000002</v>
+      </c>
+      <c r="O11" s="1">
+        <v>3.8866000000000001</v>
+      </c>
+      <c r="P11" s="1">
+        <v>3.9714999999999998</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>4.0469999999999997</v>
+      </c>
+      <c r="R11" s="1">
+        <v>4.1285999999999996</v>
+      </c>
+      <c r="S11" s="1">
+        <v>4.2176999999999998</v>
+      </c>
+      <c r="T11" s="1">
+        <v>4.3003999999999998</v>
+      </c>
+      <c r="U11" s="1">
+        <v>4.3738999999999999</v>
+      </c>
+      <c r="V11" s="1">
+        <v>4.4413</v>
+      </c>
+      <c r="W11" s="1">
+        <v>4.5106999999999999</v>
+      </c>
+      <c r="X11" s="1">
+        <v>4.5777999999999999</v>
+      </c>
+      <c r="Y11" s="1">
+        <v>4.6402000000000001</v>
+      </c>
+      <c r="Z11" s="1">
+        <v>4.6985000000000001</v>
+      </c>
+      <c r="AA11" s="1">
+        <v>4.7622</v>
+      </c>
+      <c r="AB11" s="1">
+        <v>4.8235999999999999</v>
+      </c>
+      <c r="AC11" s="1">
+        <v>4.8823999999999996</v>
+      </c>
+      <c r="AD11" s="1">
+        <v>4.9416000000000002</v>
+      </c>
+      <c r="AE11" s="1">
+        <v>4.9991000000000003</v>
+      </c>
+      <c r="AF11" s="1">
+        <v>5.0534999999999997</v>
+      </c>
+      <c r="AG11" s="1">
+        <v>5.1055000000000001</v>
+      </c>
+      <c r="AH11" s="1">
+        <v>5.1534000000000004</v>
+      </c>
+      <c r="AI11" s="1">
+        <v>5.2000999999999999</v>
+      </c>
+      <c r="AJ11" s="1">
+        <v>5.2432999999999996</v>
+      </c>
+      <c r="AK11" s="1">
+        <v>5.2869000000000002</v>
+      </c>
+      <c r="AL11" s="1">
+        <v>5.3292999999999999</v>
+      </c>
+      <c r="AM11" s="1">
+        <v>5.3691000000000004</v>
+      </c>
+      <c r="AN11" s="1">
+        <v>5.4081000000000001</v>
+      </c>
+      <c r="AO11" s="1">
+        <v>5.4466999999999999</v>
+      </c>
+      <c r="AP11" s="1">
+        <v>5.4837999999999996</v>
+      </c>
+      <c r="AQ11" s="1">
+        <v>5.5191999999999997</v>
+      </c>
+      <c r="AR11" s="1">
+        <v>5.5530999999999997</v>
+      </c>
+      <c r="AS11" s="1">
+        <v>5.5861000000000001</v>
+      </c>
+      <c r="AT11" s="1">
+        <v>5.6192000000000002</v>
+      </c>
+      <c r="AU11" s="1">
+        <v>5.6562000000000001</v>
+      </c>
+      <c r="AV11" s="1">
+        <v>5.6997999999999998</v>
+      </c>
+      <c r="AW11" s="1">
+        <v>5.7531999999999996</v>
+      </c>
+      <c r="AX11" s="1">
+        <v>5.8211000000000004</v>
+      </c>
+      <c r="AY11" s="1">
+        <v>5.9131</v>
+      </c>
+    </row>
+    <row r="12" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B12" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="28">
+        <v>6.1296999999999997</v>
+      </c>
+      <c r="G12" s="1">
+        <v>5.1375999999999999</v>
+      </c>
+      <c r="H12" s="1">
+        <v>4.6134000000000004</v>
+      </c>
+      <c r="I12" s="1">
+        <v>4.1098999999999997</v>
+      </c>
+      <c r="J12" s="1">
+        <v>3.71</v>
+      </c>
+      <c r="K12" s="1">
+        <v>3.5565000000000002</v>
+      </c>
+      <c r="L12" s="1">
+        <v>3.5167000000000002</v>
+      </c>
+      <c r="M12" s="1">
+        <v>3.5402999999999998</v>
+      </c>
+      <c r="N12" s="1">
+        <v>3.5709</v>
+      </c>
+      <c r="O12" s="1">
+        <v>3.5884999999999998</v>
+      </c>
+      <c r="P12" s="1">
+        <v>3.6080000000000001</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>3.6375999999999999</v>
+      </c>
+      <c r="R12" s="1">
+        <v>3.6827000000000001</v>
+      </c>
+      <c r="S12" s="1">
+        <v>3.7280000000000002</v>
+      </c>
+      <c r="T12" s="1">
+        <v>3.7787999999999999</v>
+      </c>
+      <c r="U12" s="1">
+        <v>3.8344</v>
+      </c>
+      <c r="V12" s="1">
+        <v>3.8938999999999999</v>
+      </c>
+      <c r="W12" s="1">
+        <v>3.9535</v>
+      </c>
+      <c r="X12" s="1">
+        <v>4.0195999999999996</v>
+      </c>
+      <c r="Y12" s="1">
+        <v>4.0932000000000004</v>
+      </c>
+      <c r="Z12" s="1">
+        <v>4.1717000000000004</v>
+      </c>
+      <c r="AA12" s="1">
+        <v>4.2478999999999996</v>
+      </c>
+      <c r="AB12" s="1">
+        <v>4.3171999999999997</v>
+      </c>
+      <c r="AC12" s="1">
+        <v>4.3818999999999999</v>
+      </c>
+      <c r="AD12" s="1">
+        <v>4.4499000000000004</v>
+      </c>
+      <c r="AE12" s="1">
+        <v>4.5179999999999998</v>
+      </c>
+      <c r="AF12" s="1">
+        <v>4.5811000000000002</v>
+      </c>
+      <c r="AG12" s="1">
+        <v>4.6414</v>
+      </c>
+      <c r="AH12" s="1">
+        <v>4.6993999999999998</v>
+      </c>
+      <c r="AI12" s="1">
+        <v>4.7577999999999996</v>
+      </c>
+      <c r="AJ12" s="1">
+        <v>4.8170999999999999</v>
+      </c>
+      <c r="AK12" s="1">
+        <v>4.8730000000000002</v>
+      </c>
+      <c r="AL12" s="1">
+        <v>4.9250999999999996</v>
+      </c>
+      <c r="AM12" s="1">
+        <v>4.9739000000000004</v>
+      </c>
+      <c r="AN12" s="1">
+        <v>5.0225999999999997</v>
+      </c>
+      <c r="AO12" s="1">
+        <v>5.0712999999999999</v>
+      </c>
+      <c r="AP12" s="1">
+        <v>5.1195000000000004</v>
+      </c>
+      <c r="AQ12" s="1">
+        <v>5.1680000000000001</v>
+      </c>
+      <c r="AR12" s="1">
+        <v>5.2160000000000002</v>
+      </c>
+      <c r="AS12" s="1">
+        <v>5.2643000000000004</v>
+      </c>
+      <c r="AT12" s="1">
+        <v>5.3171999999999997</v>
+      </c>
+      <c r="AU12" s="1">
+        <v>5.3733000000000004</v>
+      </c>
+      <c r="AV12" s="1">
+        <v>5.4317000000000002</v>
+      </c>
+      <c r="AW12" s="1">
+        <v>5.4951999999999996</v>
+      </c>
+      <c r="AX12" s="1">
+        <v>5.5696000000000003</v>
+      </c>
+      <c r="AY12" s="1">
+        <v>5.6551999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B13" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="28">
+        <v>13.6363</v>
+      </c>
+      <c r="H13" s="28">
+        <v>7.7502000000000004</v>
+      </c>
+      <c r="I13" s="1">
+        <v>5.8710000000000004</v>
+      </c>
+      <c r="J13" s="1">
+        <v>4.9850000000000003</v>
+      </c>
+      <c r="K13" s="1">
+        <v>4.4832999999999998</v>
+      </c>
+      <c r="L13" s="1">
+        <v>4.2836999999999996</v>
+      </c>
+      <c r="M13" s="1">
+        <v>4.1977000000000002</v>
+      </c>
+      <c r="N13" s="1">
+        <v>4.0949</v>
+      </c>
+      <c r="O13" s="1">
+        <v>3.9712000000000001</v>
+      </c>
+      <c r="P13" s="1">
+        <v>3.847</v>
+      </c>
+      <c r="Q13" s="1">
+        <v>3.7265999999999999</v>
+      </c>
+      <c r="R13" s="1">
+        <v>3.6303999999999998</v>
+      </c>
+      <c r="S13" s="1">
+        <v>3.5623</v>
+      </c>
+      <c r="T13" s="1">
+        <v>3.5133000000000001</v>
+      </c>
+      <c r="U13" s="1">
+        <v>3.4857999999999998</v>
+      </c>
+      <c r="V13" s="1">
+        <v>3.4771999999999998</v>
+      </c>
+      <c r="W13" s="1">
+        <v>3.4822000000000002</v>
+      </c>
+      <c r="X13" s="1">
+        <v>3.5085999999999999</v>
+      </c>
+      <c r="Y13" s="1">
+        <v>3.5472000000000001</v>
+      </c>
+      <c r="Z13" s="1">
+        <v>3.5861999999999998</v>
+      </c>
+      <c r="AA13" s="1">
+        <v>3.6337999999999999</v>
+      </c>
+      <c r="AB13" s="1">
+        <v>3.6913999999999998</v>
+      </c>
+      <c r="AC13" s="1">
+        <v>3.7462</v>
+      </c>
+      <c r="AD13" s="1">
+        <v>3.8083999999999998</v>
+      </c>
+      <c r="AE13" s="1">
+        <v>3.8702000000000001</v>
+      </c>
+      <c r="AF13" s="1">
+        <v>3.9350999999999998</v>
+      </c>
+      <c r="AG13" s="1">
+        <v>4.0026000000000002</v>
+      </c>
+      <c r="AH13" s="1">
+        <v>4.0726000000000004</v>
+      </c>
+      <c r="AI13" s="1">
+        <v>4.1437999999999997</v>
+      </c>
+      <c r="AJ13" s="1">
+        <v>4.2119</v>
+      </c>
+      <c r="AK13" s="1">
+        <v>4.2763999999999998</v>
+      </c>
+      <c r="AL13" s="1">
+        <v>4.3372999999999999</v>
+      </c>
+      <c r="AM13" s="1">
+        <v>4.3962000000000003</v>
+      </c>
+      <c r="AN13" s="1">
+        <v>4.4538000000000002</v>
+      </c>
+      <c r="AO13" s="1">
+        <v>4.5170000000000003</v>
+      </c>
+      <c r="AP13" s="1">
+        <v>4.5791000000000004</v>
+      </c>
+      <c r="AQ13" s="1">
+        <v>4.6384999999999996</v>
+      </c>
+      <c r="AR13" s="1">
+        <v>4.6952999999999996</v>
+      </c>
+      <c r="AS13" s="1">
+        <v>4.7514000000000003</v>
+      </c>
+      <c r="AT13" s="1">
+        <v>4.8090999999999999</v>
+      </c>
+      <c r="AU13" s="1">
+        <v>4.8677999999999999</v>
+      </c>
+      <c r="AV13" s="1">
+        <v>4.9291</v>
+      </c>
+      <c r="AW13" s="1">
+        <v>5.0015999999999998</v>
+      </c>
+      <c r="AX13" s="1">
+        <v>5.0843999999999996</v>
+      </c>
+      <c r="AY13" s="1">
+        <v>5.1821000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B14" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I14" s="1">
+        <v>20.132000000000001</v>
+      </c>
+      <c r="J14" s="1">
+        <v>12.0137</v>
+      </c>
+      <c r="K14" s="1">
+        <v>8.5829000000000004</v>
+      </c>
+      <c r="L14" s="1">
+        <v>6.8143000000000002</v>
+      </c>
+      <c r="M14" s="1">
+        <v>5.8784999999999998</v>
+      </c>
+      <c r="N14" s="1">
+        <v>5.3715000000000002</v>
+      </c>
+      <c r="O14" s="1">
+        <v>5.0137999999999998</v>
+      </c>
+      <c r="P14" s="1">
+        <v>4.7043999999999997</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>4.4112</v>
+      </c>
+      <c r="R14" s="1">
+        <v>4.1558999999999999</v>
+      </c>
+      <c r="S14" s="1">
+        <v>3.9337</v>
+      </c>
+      <c r="T14" s="1">
+        <v>3.7406999999999999</v>
+      </c>
+      <c r="U14" s="1">
+        <v>3.5798999999999999</v>
+      </c>
+      <c r="V14" s="1">
+        <v>3.4582999999999999</v>
+      </c>
+      <c r="W14" s="1">
+        <v>3.3816000000000002</v>
+      </c>
+      <c r="X14" s="1">
+        <v>3.3567999999999998</v>
+      </c>
+      <c r="Y14" s="1">
+        <v>3.3374999999999999</v>
+      </c>
+      <c r="Z14" s="1">
+        <v>3.3184</v>
+      </c>
+      <c r="AA14" s="1">
+        <v>3.3094000000000001</v>
+      </c>
+      <c r="AB14" s="1">
+        <v>3.3006000000000002</v>
+      </c>
+      <c r="AC14" s="1">
+        <v>3.3062999999999998</v>
+      </c>
+      <c r="AD14" s="1">
+        <v>3.3174999999999999</v>
+      </c>
+      <c r="AE14" s="1">
+        <v>3.3279999999999998</v>
+      </c>
+      <c r="AF14" s="1">
+        <v>3.3473999999999999</v>
+      </c>
+      <c r="AG14" s="1">
+        <v>3.3736000000000002</v>
+      </c>
+      <c r="AH14" s="1">
+        <v>3.4070999999999998</v>
+      </c>
+      <c r="AI14" s="1">
+        <v>3.4466000000000001</v>
+      </c>
+      <c r="AJ14" s="1">
+        <v>3.4904999999999999</v>
+      </c>
+      <c r="AK14" s="1">
+        <v>3.5434000000000001</v>
+      </c>
+      <c r="AL14" s="1">
+        <v>3.6</v>
+      </c>
+      <c r="AM14" s="1">
+        <v>3.6570999999999998</v>
+      </c>
+      <c r="AN14" s="1">
+        <v>3.714</v>
+      </c>
+      <c r="AO14" s="1">
+        <v>3.7717000000000001</v>
+      </c>
+      <c r="AP14" s="1">
+        <v>3.8300999999999998</v>
+      </c>
+      <c r="AQ14" s="1">
+        <v>3.8894000000000002</v>
+      </c>
+      <c r="AR14" s="1">
+        <v>3.9527000000000001</v>
+      </c>
+      <c r="AS14" s="1">
+        <v>4.0224000000000002</v>
+      </c>
+      <c r="AT14" s="1">
+        <v>4.0972</v>
+      </c>
+      <c r="AU14" s="1">
+        <v>4.1711999999999998</v>
+      </c>
+      <c r="AV14" s="1">
+        <v>4.2466999999999997</v>
+      </c>
+      <c r="AW14" s="1">
+        <v>4.3269000000000002</v>
+      </c>
+      <c r="AX14" s="1">
+        <v>4.4142999999999999</v>
+      </c>
+      <c r="AY14" s="1">
+        <v>4.5170000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B15" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L15" s="1">
+        <v>13.6188</v>
+      </c>
+      <c r="M15" s="1">
+        <v>10.5471</v>
+      </c>
+      <c r="N15" s="1">
+        <v>9.0310000000000006</v>
+      </c>
+      <c r="O15" s="1">
+        <v>7.7653999999999996</v>
+      </c>
+      <c r="P15" s="1">
+        <v>6.6026999999999996</v>
+      </c>
+      <c r="Q15" s="1">
+        <v>5.6485000000000003</v>
+      </c>
+      <c r="R15" s="1">
+        <v>5.0031999999999996</v>
+      </c>
+      <c r="S15" s="1">
+        <v>4.5316999999999998</v>
+      </c>
+      <c r="T15" s="1">
+        <v>4.1296999999999997</v>
+      </c>
+      <c r="U15" s="1">
+        <v>3.7978000000000001</v>
+      </c>
+      <c r="V15" s="1">
+        <v>3.5533000000000001</v>
+      </c>
+      <c r="W15" s="1">
+        <v>3.3820000000000001</v>
+      </c>
+      <c r="X15" s="1">
+        <v>3.4013</v>
+      </c>
+      <c r="Y15" s="1">
+        <v>3.4626999999999999</v>
+      </c>
+      <c r="Z15" s="1">
+        <v>3.5213999999999999</v>
+      </c>
+      <c r="AA15" s="1">
+        <v>3.5928</v>
+      </c>
+      <c r="AB15" s="1">
+        <v>3.6677</v>
+      </c>
+      <c r="AC15" s="1">
+        <v>3.7097000000000002</v>
+      </c>
+      <c r="AD15" s="1">
+        <v>3.7225000000000001</v>
+      </c>
+      <c r="AE15" s="1">
+        <v>3.6966999999999999</v>
+      </c>
+      <c r="AF15" s="1">
+        <v>3.6398000000000001</v>
+      </c>
+      <c r="AG15" s="1">
+        <v>3.5569999999999999</v>
+      </c>
+      <c r="AH15" s="1">
+        <v>3.4634</v>
+      </c>
+      <c r="AI15" s="1">
+        <v>3.3620000000000001</v>
+      </c>
+      <c r="AJ15" s="1">
+        <v>3.2608999999999999</v>
+      </c>
+      <c r="AK15" s="1">
+        <v>3.1815000000000002</v>
+      </c>
+      <c r="AL15" s="1">
+        <v>3.1299000000000001</v>
+      </c>
+      <c r="AM15" s="1">
+        <v>3.0960999999999999</v>
+      </c>
+      <c r="AN15" s="1">
+        <v>3.0819000000000001</v>
+      </c>
+      <c r="AO15" s="1">
+        <v>3.0863999999999998</v>
+      </c>
+      <c r="AP15" s="1">
+        <v>3.1137999999999999</v>
+      </c>
+      <c r="AQ15" s="1">
+        <v>3.15</v>
+      </c>
+      <c r="AR15" s="1">
+        <v>3.1941000000000002</v>
+      </c>
+      <c r="AS15" s="1">
+        <v>3.2425999999999999</v>
+      </c>
+      <c r="AT15" s="1">
+        <v>3.2995999999999999</v>
+      </c>
+      <c r="AU15" s="1">
+        <v>3.3609</v>
+      </c>
+      <c r="AV15" s="1">
+        <v>3.4264999999999999</v>
+      </c>
+      <c r="AW15" s="1">
+        <v>3.5032999999999999</v>
+      </c>
+      <c r="AX15" s="1">
+        <v>3.5941999999999998</v>
+      </c>
+      <c r="AY15" s="1">
+        <v>3.6985000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B16" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="R16" s="1">
+        <v>15.6333</v>
+      </c>
+      <c r="S16" s="1">
+        <v>14.414300000000001</v>
+      </c>
+      <c r="T16" s="1">
+        <v>13.0663</v>
+      </c>
+      <c r="U16" s="1">
+        <v>11.670199999999999</v>
+      </c>
+      <c r="V16" s="1">
+        <v>10.2904</v>
+      </c>
+      <c r="W16" s="1">
+        <v>8.9641999999999999</v>
+      </c>
+      <c r="X16" s="1">
+        <v>7.7187000000000001</v>
+      </c>
+      <c r="Y16" s="1">
+        <v>6.5884999999999998</v>
+      </c>
+      <c r="Z16" s="1">
+        <v>5.6035000000000004</v>
+      </c>
+      <c r="AA16" s="1">
+        <v>4.8209999999999997</v>
+      </c>
+      <c r="AB16" s="1">
+        <v>4.2192999999999996</v>
+      </c>
+      <c r="AC16" s="1">
+        <v>3.7688999999999999</v>
+      </c>
+      <c r="AD16" s="1">
+        <v>3.4289999999999998</v>
+      </c>
+      <c r="AE16" s="1">
+        <v>3.1920999999999999</v>
+      </c>
+      <c r="AF16" s="1">
+        <v>3.0390000000000001</v>
+      </c>
+      <c r="AG16" s="1">
+        <v>2.9691999999999998</v>
+      </c>
+      <c r="AH16" s="1">
+        <v>2.9363999999999999</v>
+      </c>
+      <c r="AI16" s="1">
+        <v>2.9159999999999999</v>
+      </c>
+      <c r="AJ16" s="1">
+        <v>2.9190999999999998</v>
+      </c>
+      <c r="AK16" s="1">
+        <v>2.9222000000000001</v>
+      </c>
+      <c r="AL16" s="1">
+        <v>2.9188000000000001</v>
+      </c>
+      <c r="AM16" s="1">
+        <v>2.9091999999999998</v>
+      </c>
+      <c r="AN16" s="1">
+        <v>2.8959000000000001</v>
+      </c>
+      <c r="AO16" s="1">
+        <v>2.8814000000000002</v>
+      </c>
+      <c r="AP16" s="1">
+        <v>2.8675999999999999</v>
+      </c>
+      <c r="AQ16" s="1">
+        <v>2.8584999999999998</v>
+      </c>
+      <c r="AR16" s="1">
+        <v>2.8557000000000001</v>
+      </c>
+      <c r="AS16" s="1">
+        <v>2.8624999999999998</v>
+      </c>
+      <c r="AT16" s="1">
+        <v>2.8757999999999999</v>
+      </c>
+      <c r="AU16" s="1">
+        <v>2.8936000000000002</v>
+      </c>
+      <c r="AV16" s="1">
+        <v>2.9165000000000001</v>
+      </c>
+      <c r="AW16" s="1">
+        <v>2.9426000000000001</v>
+      </c>
+      <c r="AX16" s="1">
+        <v>2.9811000000000001</v>
+      </c>
+      <c r="AY16" s="1">
+        <v>3.0274000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B20" s="36" t="s">
+        <v>661</v>
+      </c>
+      <c r="C20" t="s">
+        <v>662</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C3:AY16">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="10"/>
+        <cfvo type="max"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
int and ctrl validation and foPID
</commit_message>
<xml_diff>
--- a/files/Controller Design/ZNMethods_ITAE_Errors.xlsx
+++ b/files/Controller Design/ZNMethods_ITAE_Errors.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulisboa-my.sharepoint.com/personal/ist1100262_tecnico_ulisboa_pt/Documents/MEMec/Thesis/files/Controller Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="185" documentId="8_{95F32091-D855-4402-ADD3-8991BE5FE270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26216FB3-8594-41EA-B495-AA1D8894687A}"/>
+  <xr:revisionPtr revIDLastSave="221" documentId="8_{95F32091-D855-4402-ADD3-8991BE5FE270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B41285B-FE26-4CBF-88BF-4A2E64C0AD6D}"/>
   <bookViews>
-    <workbookView xWindow="-3696" yWindow="-17388" windowWidth="30936" windowHeight="17496" activeTab="3" xr2:uid="{6BCB78A0-0C46-4270-8084-079A19E30873}"/>
+    <workbookView xWindow="-3696" yWindow="-17388" windowWidth="30936" windowHeight="17496" activeTab="5" xr2:uid="{6BCB78A0-0C46-4270-8084-079A19E30873}"/>
   </bookViews>
   <sheets>
     <sheet name="CritGain" sheetId="1" r:id="rId1"/>
     <sheet name="PID_Models" sheetId="3" r:id="rId2"/>
     <sheet name="Gains" sheetId="5" r:id="rId3"/>
     <sheet name="PID_Models_Noise" sheetId="6" r:id="rId4"/>
+    <sheet name="id_ctrl_val" sheetId="7" r:id="rId5"/>
+    <sheet name="id_ctrl_noise" sheetId="8" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1332" uniqueCount="665">
   <si>
     <t>ν/ζ</t>
   </si>
@@ -2031,6 +2033,12 @@
   </si>
   <si>
     <t>Simulations kept over 30 seconds</t>
+  </si>
+  <si>
+    <t>need to add Wcp fallback</t>
+  </si>
+  <si>
+    <t>Noise level 0.03</t>
   </si>
 </sst>
 </file>
@@ -2509,6 +2517,7 @@
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2527,7 +2536,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2929,28 +2937,28 @@
   <sheetData>
     <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="36"/>
     </row>
     <row r="3" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="33"/>
     </row>
     <row r="5" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="33"/>
     </row>
     <row r="7" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="20" t="s">
@@ -3328,11 +3336,11 @@
     </row>
     <row r="18" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="19" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="31"/>
-      <c r="D19" s="32"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="33"/>
     </row>
     <row r="20" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="20" t="s">
@@ -3710,11 +3718,11 @@
     </row>
     <row r="31" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="32" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="30" t="s">
+      <c r="B32" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="31"/>
-      <c r="D32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="33"/>
     </row>
     <row r="33" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="20" t="s">
@@ -22373,7 +22381,7 @@
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="30" t="s">
         <v>661</v>
       </c>
       <c r="C20" t="s">
@@ -22395,4 +22403,4325 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E237936-F695-4675-B42C-B0BF8FA4F476}">
+  <dimension ref="B1:AY15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="51" width="6.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="K2" s="1">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M2" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="N2" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="O2" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="P2" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="R2" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="S2" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="T2" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="U2" s="1">
+        <v>2</v>
+      </c>
+      <c r="V2" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="W2" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="X2" s="1">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>2.4</v>
+      </c>
+      <c r="Z2" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="AA2" s="1">
+        <v>2.6</v>
+      </c>
+      <c r="AB2" s="1">
+        <v>2.7</v>
+      </c>
+      <c r="AC2" s="1">
+        <v>2.8</v>
+      </c>
+      <c r="AD2" s="1">
+        <v>2.9</v>
+      </c>
+      <c r="AE2" s="1">
+        <v>3</v>
+      </c>
+      <c r="AF2" s="1">
+        <v>3.1</v>
+      </c>
+      <c r="AG2" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="AH2" s="1">
+        <v>3.3</v>
+      </c>
+      <c r="AI2" s="1">
+        <v>3.4</v>
+      </c>
+      <c r="AJ2" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="AK2" s="1">
+        <v>3.6</v>
+      </c>
+      <c r="AL2" s="1">
+        <v>3.7</v>
+      </c>
+      <c r="AM2" s="1">
+        <v>3.8</v>
+      </c>
+      <c r="AN2" s="1">
+        <v>3.9</v>
+      </c>
+      <c r="AO2" s="1">
+        <v>4</v>
+      </c>
+      <c r="AP2" s="1">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AQ2" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="AR2" s="1">
+        <v>4.3</v>
+      </c>
+      <c r="AS2" s="1">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AT2" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="AU2" s="1">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AV2" s="1">
+        <v>4.7</v>
+      </c>
+      <c r="AW2" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="AX2" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="AY2" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B3" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.4713</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.1545</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.15390000000000001</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0.21429999999999999</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0.21379999999999999</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0.24809999999999999</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0.29780000000000001</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0.3503</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0.40450000000000003</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0.53539999999999999</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0.61499999999999999</v>
+      </c>
+      <c r="P3" s="1">
+        <v>0.70140000000000002</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>0.79500000000000004</v>
+      </c>
+      <c r="R3" s="1">
+        <v>0.61360000000000003</v>
+      </c>
+      <c r="S3" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="T3" s="1">
+        <v>0.58840000000000003</v>
+      </c>
+      <c r="U3" s="1">
+        <v>0.57620000000000005</v>
+      </c>
+      <c r="V3" s="1">
+        <v>0.89529999999999998</v>
+      </c>
+      <c r="W3" s="1">
+        <v>0.78749999999999998</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AG3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AL3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AM3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AN3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AO3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AP3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AQ3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AR3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AS3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AT3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AU3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AV3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AW3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AX3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AY3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B4" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.97740000000000005</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.3125</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.1119</v>
+      </c>
+      <c r="F4" s="1">
+        <v>7.5700000000000003E-2</v>
+      </c>
+      <c r="G4" s="1">
+        <v>8.6800000000000002E-2</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0.11020000000000001</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0.1201</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0.124</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0.13089999999999999</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0.14069999999999999</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0.1532</v>
+      </c>
+      <c r="N4" s="1">
+        <v>0.1681</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0.185</v>
+      </c>
+      <c r="P4" s="1">
+        <v>0.2031</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>0.2218</v>
+      </c>
+      <c r="R4" s="1">
+        <v>0.2409</v>
+      </c>
+      <c r="S4" s="1">
+        <v>0.26050000000000001</v>
+      </c>
+      <c r="T4" s="1">
+        <v>0.28129999999999999</v>
+      </c>
+      <c r="U4" s="1">
+        <v>0.30420000000000003</v>
+      </c>
+      <c r="V4" s="1">
+        <v>0.33050000000000002</v>
+      </c>
+      <c r="W4" s="1">
+        <v>0.3619</v>
+      </c>
+      <c r="X4" s="1">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>0.37859999999999999</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>0.39960000000000001</v>
+      </c>
+      <c r="AA4" s="1">
+        <v>0.42459999999999998</v>
+      </c>
+      <c r="AB4" s="1">
+        <v>0.4526</v>
+      </c>
+      <c r="AC4" s="1">
+        <v>0.48220000000000002</v>
+      </c>
+      <c r="AD4" s="1">
+        <v>0.51219999999999999</v>
+      </c>
+      <c r="AE4" s="1">
+        <v>0.54110000000000003</v>
+      </c>
+      <c r="AF4" s="1">
+        <v>0.56810000000000005</v>
+      </c>
+      <c r="AG4" s="1">
+        <v>0.59319999999999995</v>
+      </c>
+      <c r="AH4" s="1">
+        <v>0.61729999999999996</v>
+      </c>
+      <c r="AI4" s="1">
+        <v>0.64319999999999999</v>
+      </c>
+      <c r="AJ4" s="1">
+        <v>0.67510000000000003</v>
+      </c>
+      <c r="AK4" s="1">
+        <v>0.71819999999999995</v>
+      </c>
+      <c r="AL4" s="1">
+        <v>0.77690000000000003</v>
+      </c>
+      <c r="AM4" s="1">
+        <v>0.85219999999999996</v>
+      </c>
+      <c r="AN4" s="1">
+        <v>0.94010000000000005</v>
+      </c>
+      <c r="AO4" s="1">
+        <v>1.0319</v>
+      </c>
+      <c r="AP4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AQ4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AR4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AS4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AT4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AU4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AV4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AW4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AX4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AY4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B5" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2.2170000000000001</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.65310000000000001</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.29580000000000001</v>
+      </c>
+      <c r="F5" s="1">
+        <v>2.4899999999999999E-2</v>
+      </c>
+      <c r="G5" s="1">
+        <v>3.7699999999999997E-2</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3.9300000000000002E-2</v>
+      </c>
+      <c r="I5" s="1">
+        <v>5.16E-2</v>
+      </c>
+      <c r="J5" s="1">
+        <v>6.1600000000000002E-2</v>
+      </c>
+      <c r="K5" s="1">
+        <v>6.8500000000000005E-2</v>
+      </c>
+      <c r="L5" s="1">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="M5" s="1">
+        <v>8.2799999999999999E-2</v>
+      </c>
+      <c r="N5" s="1">
+        <v>9.2399999999999996E-2</v>
+      </c>
+      <c r="O5" s="1">
+        <v>0.1032</v>
+      </c>
+      <c r="P5" s="1">
+        <v>0.1143</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="R5" s="1">
+        <v>0.13519999999999999</v>
+      </c>
+      <c r="S5" s="1">
+        <v>0.1452</v>
+      </c>
+      <c r="T5" s="1">
+        <v>0.15570000000000001</v>
+      </c>
+      <c r="U5" s="1">
+        <v>0.1676</v>
+      </c>
+      <c r="V5" s="1">
+        <v>0.2298</v>
+      </c>
+      <c r="W5" s="1">
+        <v>0.22359999999999999</v>
+      </c>
+      <c r="X5" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>0.21929999999999999</v>
+      </c>
+      <c r="Z5" s="1">
+        <v>0.2218</v>
+      </c>
+      <c r="AA5" s="1">
+        <v>0.22770000000000001</v>
+      </c>
+      <c r="AB5" s="1">
+        <v>0.2369</v>
+      </c>
+      <c r="AC5" s="1">
+        <v>0.24970000000000001</v>
+      </c>
+      <c r="AD5" s="1">
+        <v>0.26619999999999999</v>
+      </c>
+      <c r="AE5" s="1">
+        <v>0.28710000000000002</v>
+      </c>
+      <c r="AF5" s="1">
+        <v>0.31380000000000002</v>
+      </c>
+      <c r="AG5" s="1">
+        <v>0.3478</v>
+      </c>
+      <c r="AH5" s="1">
+        <v>0.39090000000000003</v>
+      </c>
+      <c r="AI5" s="1">
+        <v>0.44490000000000002</v>
+      </c>
+      <c r="AJ5" s="1">
+        <v>0.51100000000000001</v>
+      </c>
+      <c r="AK5" s="1">
+        <v>0.58979999999999999</v>
+      </c>
+      <c r="AL5" s="1">
+        <v>0.67989999999999995</v>
+      </c>
+      <c r="AM5" s="1">
+        <v>0.77859999999999996</v>
+      </c>
+      <c r="AN5" s="1">
+        <v>0.87549999999999994</v>
+      </c>
+      <c r="AO5" s="1">
+        <v>0.96309999999999996</v>
+      </c>
+      <c r="AP5" s="1">
+        <v>1.0374000000000001</v>
+      </c>
+      <c r="AQ5" s="1">
+        <v>1.0952</v>
+      </c>
+      <c r="AR5" s="1">
+        <v>1.1339999999999999</v>
+      </c>
+      <c r="AS5" s="1">
+        <v>1.1516</v>
+      </c>
+      <c r="AT5" s="1">
+        <v>1.1469</v>
+      </c>
+      <c r="AU5" s="1">
+        <v>1.119</v>
+      </c>
+      <c r="AV5" s="1">
+        <v>1.0671999999999999</v>
+      </c>
+      <c r="AW5" s="1">
+        <v>0.99170000000000003</v>
+      </c>
+      <c r="AX5" s="1">
+        <v>0.89259999999999995</v>
+      </c>
+      <c r="AY5" s="1">
+        <v>0.77559999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B6" s="1">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3.4996999999999998</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1.8875</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.56779999999999997</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.42959999999999998</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0.17469999999999999</v>
+      </c>
+      <c r="H6" s="1">
+        <v>5.0599999999999999E-2</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="J6" s="1">
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1.0200000000000001E-2</v>
+      </c>
+      <c r="L6" s="1">
+        <v>1.46E-2</v>
+      </c>
+      <c r="M6" s="1">
+        <v>2.0199999999999999E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>2.92E-2</v>
+      </c>
+      <c r="O6" s="1">
+        <v>4.2099999999999999E-2</v>
+      </c>
+      <c r="P6" s="1">
+        <v>5.79E-2</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>7.46E-2</v>
+      </c>
+      <c r="R6" s="1">
+        <v>9.1399999999999995E-2</v>
+      </c>
+      <c r="S6" s="1">
+        <v>0.1095</v>
+      </c>
+      <c r="T6" s="1">
+        <v>0.1711</v>
+      </c>
+      <c r="U6" s="1">
+        <v>0.17910000000000001</v>
+      </c>
+      <c r="V6" s="1">
+        <v>0.18640000000000001</v>
+      </c>
+      <c r="W6" s="1">
+        <v>0.19489999999999999</v>
+      </c>
+      <c r="X6" s="1">
+        <v>0.20630000000000001</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>0.22170000000000001</v>
+      </c>
+      <c r="Z6" s="1">
+        <v>0.24229999999999999</v>
+      </c>
+      <c r="AA6" s="1">
+        <v>0.26879999999999998</v>
+      </c>
+      <c r="AB6" s="1">
+        <v>0.3019</v>
+      </c>
+      <c r="AC6" s="1">
+        <v>0.34189999999999998</v>
+      </c>
+      <c r="AD6" s="1">
+        <v>0.38869999999999999</v>
+      </c>
+      <c r="AE6" s="1">
+        <v>0.44190000000000002</v>
+      </c>
+      <c r="AF6" s="1">
+        <v>0.50039999999999996</v>
+      </c>
+      <c r="AG6" s="1">
+        <v>0.56320000000000003</v>
+      </c>
+      <c r="AH6" s="1">
+        <v>0.62839999999999996</v>
+      </c>
+      <c r="AI6" s="1">
+        <v>0.69410000000000005</v>
+      </c>
+      <c r="AJ6" s="1">
+        <v>0.75839999999999996</v>
+      </c>
+      <c r="AK6" s="1">
+        <v>0.81930000000000003</v>
+      </c>
+      <c r="AL6" s="1">
+        <v>0.87490000000000001</v>
+      </c>
+      <c r="AM6" s="1">
+        <v>0.92379999999999995</v>
+      </c>
+      <c r="AN6" s="1">
+        <v>0.96479999999999999</v>
+      </c>
+      <c r="AO6" s="1">
+        <v>0.99680000000000002</v>
+      </c>
+      <c r="AP6" s="1">
+        <v>1.0192000000000001</v>
+      </c>
+      <c r="AQ6" s="1">
+        <v>1.0316000000000001</v>
+      </c>
+      <c r="AR6" s="1">
+        <v>1.0339</v>
+      </c>
+      <c r="AS6" s="1">
+        <v>1.0262</v>
+      </c>
+      <c r="AT6" s="1">
+        <v>1.0086999999999999</v>
+      </c>
+      <c r="AU6" s="1">
+        <v>0.98180000000000001</v>
+      </c>
+      <c r="AV6" s="1">
+        <v>0.94579999999999997</v>
+      </c>
+      <c r="AW6" s="1">
+        <v>0.90149999999999997</v>
+      </c>
+      <c r="AX6" s="1">
+        <v>0.84930000000000005</v>
+      </c>
+      <c r="AY6" s="1">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="7" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B7" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C7" s="1">
+        <v>3.6701000000000001</v>
+      </c>
+      <c r="D7" s="1">
+        <v>3.8868999999999998</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1.9161999999999999</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.56740000000000002</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0.69479999999999997</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0.52810000000000001</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.31659999999999999</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0.22459999999999999</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0.20300000000000001</v>
+      </c>
+      <c r="L7" s="1">
+        <v>5.8200000000000002E-2</v>
+      </c>
+      <c r="M7" s="1">
+        <v>6.25E-2</v>
+      </c>
+      <c r="N7" s="1">
+        <v>7.1400000000000005E-2</v>
+      </c>
+      <c r="O7" s="1">
+        <v>8.1600000000000006E-2</v>
+      </c>
+      <c r="P7" s="1">
+        <v>9.0300000000000005E-2</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>9.6299999999999997E-2</v>
+      </c>
+      <c r="R7" s="1">
+        <v>0.1014</v>
+      </c>
+      <c r="S7" s="1">
+        <v>0.10829999999999999</v>
+      </c>
+      <c r="T7" s="1">
+        <v>0.1179</v>
+      </c>
+      <c r="U7" s="1">
+        <v>0.13059999999999999</v>
+      </c>
+      <c r="V7" s="1">
+        <v>0.1396</v>
+      </c>
+      <c r="W7" s="1">
+        <v>0.14879999999999999</v>
+      </c>
+      <c r="X7" s="1">
+        <v>0.15759999999999999</v>
+      </c>
+      <c r="Y7" s="1">
+        <v>0.1671</v>
+      </c>
+      <c r="Z7" s="1">
+        <v>0.17799999999999999</v>
+      </c>
+      <c r="AA7" s="1">
+        <v>0.1908</v>
+      </c>
+      <c r="AB7" s="1">
+        <v>0.2059</v>
+      </c>
+      <c r="AC7" s="1">
+        <v>0.2235</v>
+      </c>
+      <c r="AD7" s="1">
+        <v>0.24379999999999999</v>
+      </c>
+      <c r="AE7" s="1">
+        <v>0.26690000000000003</v>
+      </c>
+      <c r="AF7" s="1">
+        <v>0.29249999999999998</v>
+      </c>
+      <c r="AG7" s="1">
+        <v>0.32029999999999997</v>
+      </c>
+      <c r="AH7" s="1">
+        <v>0.3498</v>
+      </c>
+      <c r="AI7" s="1">
+        <v>0.38040000000000002</v>
+      </c>
+      <c r="AJ7" s="1">
+        <v>0.41139999999999999</v>
+      </c>
+      <c r="AK7" s="1">
+        <v>0.44219999999999998</v>
+      </c>
+      <c r="AL7" s="1">
+        <v>0.47220000000000001</v>
+      </c>
+      <c r="AM7" s="1">
+        <v>0.501</v>
+      </c>
+      <c r="AN7" s="1">
+        <v>0.52810000000000001</v>
+      </c>
+      <c r="AO7" s="1">
+        <v>0.55300000000000005</v>
+      </c>
+      <c r="AP7" s="1">
+        <v>0.57550000000000001</v>
+      </c>
+      <c r="AQ7" s="1">
+        <v>0.59540000000000004</v>
+      </c>
+      <c r="AR7" s="1">
+        <v>0.61240000000000006</v>
+      </c>
+      <c r="AS7" s="1">
+        <v>0.62660000000000005</v>
+      </c>
+      <c r="AT7" s="1">
+        <v>0.63780000000000003</v>
+      </c>
+      <c r="AU7" s="1">
+        <v>0.64610000000000001</v>
+      </c>
+      <c r="AV7" s="1">
+        <v>0.65159999999999996</v>
+      </c>
+      <c r="AW7" s="1">
+        <v>0.65439999999999998</v>
+      </c>
+      <c r="AX7" s="1">
+        <v>0.65459999999999996</v>
+      </c>
+      <c r="AY7" s="1">
+        <v>0.65249999999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B8" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="C8" s="1">
+        <v>3.8708999999999998</v>
+      </c>
+      <c r="D8" s="1">
+        <v>3.8222</v>
+      </c>
+      <c r="E8" s="1">
+        <v>4.1124000000000001</v>
+      </c>
+      <c r="F8" s="1">
+        <v>2.2105999999999999</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1.3871</v>
+      </c>
+      <c r="H8" s="1">
+        <v>1.2366999999999999</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0.92830000000000001</v>
+      </c>
+      <c r="J8" s="1">
+        <v>0.59179999999999999</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0.4002</v>
+      </c>
+      <c r="L8" s="1">
+        <v>0.29799999999999999</v>
+      </c>
+      <c r="M8" s="1">
+        <v>0.24210000000000001</v>
+      </c>
+      <c r="N8" s="1">
+        <v>0.2137</v>
+      </c>
+      <c r="O8" s="1">
+        <v>0.19739999999999999</v>
+      </c>
+      <c r="P8" s="1">
+        <v>0.1867</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>0.191</v>
+      </c>
+      <c r="R8" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="S8" s="1">
+        <v>0.19800000000000001</v>
+      </c>
+      <c r="T8" s="1">
+        <v>0.20549999999999999</v>
+      </c>
+      <c r="U8" s="1">
+        <v>0.2114</v>
+      </c>
+      <c r="V8" s="1">
+        <v>0.21529999999999999</v>
+      </c>
+      <c r="W8" s="1">
+        <v>0.25559999999999999</v>
+      </c>
+      <c r="X8" s="1">
+        <v>0.25409999999999999</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>0.2576</v>
+      </c>
+      <c r="Z8" s="1">
+        <v>0.26929999999999998</v>
+      </c>
+      <c r="AA8" s="1">
+        <v>0.28220000000000001</v>
+      </c>
+      <c r="AB8" s="1">
+        <v>0.29070000000000001</v>
+      </c>
+      <c r="AC8" s="1">
+        <v>0.30270000000000002</v>
+      </c>
+      <c r="AD8" s="1">
+        <v>0.31619999999999998</v>
+      </c>
+      <c r="AE8" s="1">
+        <v>0.3322</v>
+      </c>
+      <c r="AF8" s="1">
+        <v>0.3538</v>
+      </c>
+      <c r="AG8" s="1">
+        <v>0.38679999999999998</v>
+      </c>
+      <c r="AH8" s="1">
+        <v>0.441</v>
+      </c>
+      <c r="AI8" s="1">
+        <v>0.52359999999999995</v>
+      </c>
+      <c r="AJ8" s="1">
+        <v>0.62260000000000004</v>
+      </c>
+      <c r="AK8" s="1">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="AL8" s="1">
+        <v>0.62509999999999999</v>
+      </c>
+      <c r="AM8" s="1">
+        <v>0.72750000000000004</v>
+      </c>
+      <c r="AN8" s="1">
+        <v>0.65480000000000005</v>
+      </c>
+      <c r="AO8" s="1">
+        <v>0.73839999999999995</v>
+      </c>
+      <c r="AP8" s="1">
+        <v>0.48830000000000001</v>
+      </c>
+      <c r="AQ8" s="1">
+        <v>0.57130000000000003</v>
+      </c>
+      <c r="AR8" s="1">
+        <v>0.67900000000000005</v>
+      </c>
+      <c r="AS8" s="1">
+        <v>0.75749999999999995</v>
+      </c>
+      <c r="AT8" s="1">
+        <v>0.64810000000000001</v>
+      </c>
+      <c r="AU8" s="1">
+        <v>0.55259999999999998</v>
+      </c>
+      <c r="AV8" s="1">
+        <v>0.65490000000000004</v>
+      </c>
+      <c r="AW8" s="1">
+        <v>0.71140000000000003</v>
+      </c>
+      <c r="AX8" s="1">
+        <v>0.7056</v>
+      </c>
+      <c r="AY8" s="1">
+        <v>0.60619999999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B9" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="1">
+        <v>4.0770999999999997</v>
+      </c>
+      <c r="E9" s="1">
+        <v>3.6833</v>
+      </c>
+      <c r="F9" s="1">
+        <v>3.8306</v>
+      </c>
+      <c r="G9" s="1">
+        <v>3.5510000000000002</v>
+      </c>
+      <c r="H9" s="1">
+        <v>2.6949000000000001</v>
+      </c>
+      <c r="I9" s="1">
+        <v>2.1476999999999999</v>
+      </c>
+      <c r="J9" s="1">
+        <v>1.5486</v>
+      </c>
+      <c r="K9" s="1">
+        <v>1.048</v>
+      </c>
+      <c r="L9" s="1">
+        <v>0.75590000000000002</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0.54390000000000005</v>
+      </c>
+      <c r="N9" s="1">
+        <v>0.47539999999999999</v>
+      </c>
+      <c r="O9" s="1">
+        <v>0.38650000000000001</v>
+      </c>
+      <c r="P9" s="1">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>0.28970000000000001</v>
+      </c>
+      <c r="R9" s="1">
+        <v>0.29139999999999999</v>
+      </c>
+      <c r="S9" s="1">
+        <v>0.2944</v>
+      </c>
+      <c r="T9" s="1">
+        <v>0.309</v>
+      </c>
+      <c r="U9" s="1">
+        <v>0.30249999999999999</v>
+      </c>
+      <c r="V9" s="1">
+        <v>0.37469999999999998</v>
+      </c>
+      <c r="W9" s="1">
+        <v>0.36349999999999999</v>
+      </c>
+      <c r="X9" s="1">
+        <v>0.36270000000000002</v>
+      </c>
+      <c r="Y9" s="1">
+        <v>0.3644</v>
+      </c>
+      <c r="Z9" s="1">
+        <v>0.36730000000000002</v>
+      </c>
+      <c r="AA9" s="1">
+        <v>0.37059999999999998</v>
+      </c>
+      <c r="AB9" s="1">
+        <v>0.37369999999999998</v>
+      </c>
+      <c r="AC9" s="1">
+        <v>0.37669999999999998</v>
+      </c>
+      <c r="AD9" s="1">
+        <v>0.3856</v>
+      </c>
+      <c r="AE9" s="1">
+        <v>0.40600000000000003</v>
+      </c>
+      <c r="AF9" s="1">
+        <v>0.40689999999999998</v>
+      </c>
+      <c r="AG9" s="1">
+        <v>0.47149999999999997</v>
+      </c>
+      <c r="AH9" s="1">
+        <v>0.43430000000000002</v>
+      </c>
+      <c r="AI9" s="1">
+        <v>0.53569999999999995</v>
+      </c>
+      <c r="AJ9" s="1">
+        <v>0.49509999999999998</v>
+      </c>
+      <c r="AK9" s="1">
+        <v>0.47720000000000001</v>
+      </c>
+      <c r="AL9" s="1">
+        <v>0.59909999999999997</v>
+      </c>
+      <c r="AM9" s="1">
+        <v>0.57609999999999995</v>
+      </c>
+      <c r="AN9" s="1">
+        <v>0.55940000000000001</v>
+      </c>
+      <c r="AO9" s="1">
+        <v>0.55369999999999997</v>
+      </c>
+      <c r="AP9" s="1">
+        <v>0.66859999999999997</v>
+      </c>
+      <c r="AQ9" s="1">
+        <v>0.66180000000000005</v>
+      </c>
+      <c r="AR9" s="1">
+        <v>0.65610000000000002</v>
+      </c>
+      <c r="AS9" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="AT9" s="1">
+        <v>0.64839999999999998</v>
+      </c>
+      <c r="AU9" s="1">
+        <v>0.65200000000000002</v>
+      </c>
+      <c r="AV9" s="1">
+        <v>0.65920000000000001</v>
+      </c>
+      <c r="AW9" s="1">
+        <v>0.67410000000000003</v>
+      </c>
+      <c r="AX9" s="1">
+        <v>0.70660000000000001</v>
+      </c>
+      <c r="AY9" s="1">
+        <v>0.71289999999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B10" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="1">
+        <v>4.1971999999999996</v>
+      </c>
+      <c r="F10" s="1">
+        <v>3.6046999999999998</v>
+      </c>
+      <c r="G10" s="1">
+        <v>3.3809</v>
+      </c>
+      <c r="H10" s="1">
+        <v>3.4356</v>
+      </c>
+      <c r="I10" s="1">
+        <v>3.3374000000000001</v>
+      </c>
+      <c r="J10" s="1">
+        <v>2.8334999999999999</v>
+      </c>
+      <c r="K10" s="1">
+        <v>1.9409000000000001</v>
+      </c>
+      <c r="L10" s="1">
+        <v>1.6054999999999999</v>
+      </c>
+      <c r="M10" s="1">
+        <v>1.0538000000000001</v>
+      </c>
+      <c r="N10" s="1">
+        <v>0.69920000000000004</v>
+      </c>
+      <c r="O10" s="1">
+        <v>0.49859999999999999</v>
+      </c>
+      <c r="P10" s="1">
+        <v>0.4073</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>0.57189999999999996</v>
+      </c>
+      <c r="R10" s="1">
+        <v>0.57150000000000001</v>
+      </c>
+      <c r="S10" s="1">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="T10" s="1">
+        <v>0.51</v>
+      </c>
+      <c r="U10" s="1">
+        <v>0.61439999999999995</v>
+      </c>
+      <c r="V10" s="1">
+        <v>0.54430000000000001</v>
+      </c>
+      <c r="W10" s="1">
+        <v>0.55730000000000002</v>
+      </c>
+      <c r="X10" s="1">
+        <v>0.4985</v>
+      </c>
+      <c r="Y10" s="1">
+        <v>0.46260000000000001</v>
+      </c>
+      <c r="Z10" s="1">
+        <v>0.4587</v>
+      </c>
+      <c r="AA10" s="1">
+        <v>0.44869999999999999</v>
+      </c>
+      <c r="AB10" s="1">
+        <v>0.43869999999999998</v>
+      </c>
+      <c r="AC10" s="1">
+        <v>0.47099999999999997</v>
+      </c>
+      <c r="AD10" s="1">
+        <v>0.45910000000000001</v>
+      </c>
+      <c r="AE10" s="1">
+        <v>0.45069999999999999</v>
+      </c>
+      <c r="AF10" s="1">
+        <v>0.54730000000000001</v>
+      </c>
+      <c r="AG10" s="1">
+        <v>0.54590000000000005</v>
+      </c>
+      <c r="AH10" s="1">
+        <v>0.54990000000000006</v>
+      </c>
+      <c r="AI10" s="1">
+        <v>0.55920000000000003</v>
+      </c>
+      <c r="AJ10" s="1">
+        <v>0.57379999999999998</v>
+      </c>
+      <c r="AK10" s="1">
+        <v>0.59350000000000003</v>
+      </c>
+      <c r="AL10" s="1">
+        <v>0.61729999999999996</v>
+      </c>
+      <c r="AM10" s="1">
+        <v>0.64339999999999997</v>
+      </c>
+      <c r="AN10" s="1">
+        <v>0.66749999999999998</v>
+      </c>
+      <c r="AO10" s="1">
+        <v>0.6825</v>
+      </c>
+      <c r="AP10" s="1">
+        <v>0.61529999999999996</v>
+      </c>
+      <c r="AQ10" s="1">
+        <v>0.64959999999999996</v>
+      </c>
+      <c r="AR10" s="1">
+        <v>0.66769999999999996</v>
+      </c>
+      <c r="AS10" s="1">
+        <v>0.65129999999999999</v>
+      </c>
+      <c r="AT10" s="1">
+        <v>0.65059999999999996</v>
+      </c>
+      <c r="AU10" s="1">
+        <v>0.64649999999999996</v>
+      </c>
+      <c r="AV10" s="1">
+        <v>0.59770000000000001</v>
+      </c>
+      <c r="AW10" s="1">
+        <v>0.6341</v>
+      </c>
+      <c r="AX10" s="1">
+        <v>0.62180000000000002</v>
+      </c>
+      <c r="AY10" s="1">
+        <v>0.62290000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B11" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="28">
+        <v>5.0037000000000003</v>
+      </c>
+      <c r="G11" s="1">
+        <v>3.8614999999999999</v>
+      </c>
+      <c r="H11" s="1">
+        <v>3.0076999999999998</v>
+      </c>
+      <c r="I11" s="1">
+        <v>2.4432</v>
+      </c>
+      <c r="J11" s="1">
+        <v>2.3041999999999998</v>
+      </c>
+      <c r="K11" s="1">
+        <v>1.7255</v>
+      </c>
+      <c r="L11" s="1">
+        <v>1.9196</v>
+      </c>
+      <c r="M11" s="1">
+        <v>1.2383</v>
+      </c>
+      <c r="N11" s="1">
+        <v>0.72760000000000002</v>
+      </c>
+      <c r="O11" s="1">
+        <v>0.56569999999999998</v>
+      </c>
+      <c r="P11" s="1">
+        <v>1.0287999999999999</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>1.0107999999999999</v>
+      </c>
+      <c r="R11" s="1">
+        <v>0.94379999999999997</v>
+      </c>
+      <c r="S11" s="1">
+        <v>0.84560000000000002</v>
+      </c>
+      <c r="T11" s="1">
+        <v>0.87819999999999998</v>
+      </c>
+      <c r="U11" s="1">
+        <v>0.74250000000000005</v>
+      </c>
+      <c r="V11" s="1">
+        <v>0.63480000000000003</v>
+      </c>
+      <c r="W11" s="1">
+        <v>0.70930000000000004</v>
+      </c>
+      <c r="X11" s="1">
+        <v>0.60540000000000005</v>
+      </c>
+      <c r="Y11" s="1">
+        <v>0.53700000000000003</v>
+      </c>
+      <c r="Z11" s="1">
+        <v>0.56169999999999998</v>
+      </c>
+      <c r="AA11" s="1">
+        <v>0.51370000000000005</v>
+      </c>
+      <c r="AB11" s="1">
+        <v>0.52090000000000003</v>
+      </c>
+      <c r="AC11" s="1">
+        <v>0.50649999999999995</v>
+      </c>
+      <c r="AD11" s="1">
+        <v>0.501</v>
+      </c>
+      <c r="AE11" s="1">
+        <v>0.53610000000000002</v>
+      </c>
+      <c r="AF11" s="1">
+        <v>0.52329999999999999</v>
+      </c>
+      <c r="AG11" s="1">
+        <v>0.51429999999999998</v>
+      </c>
+      <c r="AH11" s="1">
+        <v>0.64670000000000005</v>
+      </c>
+      <c r="AI11" s="1">
+        <v>0.60250000000000004</v>
+      </c>
+      <c r="AJ11" s="1">
+        <v>0.59630000000000005</v>
+      </c>
+      <c r="AK11" s="1">
+        <v>0.59770000000000001</v>
+      </c>
+      <c r="AL11" s="1">
+        <v>0.60289999999999999</v>
+      </c>
+      <c r="AM11" s="1">
+        <v>0.61180000000000001</v>
+      </c>
+      <c r="AN11" s="1">
+        <v>0.62409999999999999</v>
+      </c>
+      <c r="AO11" s="1">
+        <v>0.63919999999999999</v>
+      </c>
+      <c r="AP11" s="1">
+        <v>0.65580000000000005</v>
+      </c>
+      <c r="AQ11" s="1">
+        <v>0.67159999999999997</v>
+      </c>
+      <c r="AR11" s="1">
+        <v>0.68269999999999997</v>
+      </c>
+      <c r="AS11" s="1">
+        <v>0.68600000000000005</v>
+      </c>
+      <c r="AT11" s="1">
+        <v>0.71150000000000002</v>
+      </c>
+      <c r="AU11" s="1">
+        <v>0.66469999999999996</v>
+      </c>
+      <c r="AV11" s="1">
+        <v>0.67369999999999997</v>
+      </c>
+      <c r="AW11" s="1">
+        <v>0.65580000000000005</v>
+      </c>
+      <c r="AX11" s="1">
+        <v>0.66990000000000005</v>
+      </c>
+      <c r="AY11" s="1">
+        <v>0.66190000000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B12" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="28">
+        <v>6.8117000000000001</v>
+      </c>
+      <c r="H12" s="28">
+        <v>4.9020000000000001</v>
+      </c>
+      <c r="I12" s="1">
+        <v>3.5665</v>
+      </c>
+      <c r="J12" s="1">
+        <v>2.4251999999999998</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1.7601</v>
+      </c>
+      <c r="L12" s="1">
+        <v>1.4361999999999999</v>
+      </c>
+      <c r="M12" s="1">
+        <v>1.3228</v>
+      </c>
+      <c r="N12" s="1">
+        <v>2.1444000000000001</v>
+      </c>
+      <c r="O12" s="1">
+        <v>1.9611000000000001</v>
+      </c>
+      <c r="P12" s="1">
+        <v>1.8125</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>1.6415</v>
+      </c>
+      <c r="R12" s="1">
+        <v>1.5130999999999999</v>
+      </c>
+      <c r="S12" s="1">
+        <v>1.4021999999999999</v>
+      </c>
+      <c r="T12" s="1">
+        <v>0.85309999999999997</v>
+      </c>
+      <c r="U12" s="1">
+        <v>0.86080000000000001</v>
+      </c>
+      <c r="V12" s="1">
+        <v>0.84150000000000003</v>
+      </c>
+      <c r="W12" s="1">
+        <v>0.80289999999999995</v>
+      </c>
+      <c r="X12" s="1">
+        <v>0.75670000000000004</v>
+      </c>
+      <c r="Y12" s="1">
+        <v>0.69989999999999997</v>
+      </c>
+      <c r="Z12" s="1">
+        <v>0.63360000000000005</v>
+      </c>
+      <c r="AA12" s="1">
+        <v>0.56950000000000001</v>
+      </c>
+      <c r="AB12" s="1">
+        <v>0.50860000000000005</v>
+      </c>
+      <c r="AC12" s="1">
+        <v>0.4869</v>
+      </c>
+      <c r="AD12" s="1">
+        <v>0.51580000000000004</v>
+      </c>
+      <c r="AE12" s="1">
+        <v>0.54559999999999997</v>
+      </c>
+      <c r="AF12" s="1">
+        <v>0.50219999999999998</v>
+      </c>
+      <c r="AG12" s="1">
+        <v>0.58830000000000005</v>
+      </c>
+      <c r="AH12" s="1">
+        <v>0.52129999999999999</v>
+      </c>
+      <c r="AI12" s="1">
+        <v>0.5595</v>
+      </c>
+      <c r="AJ12" s="1">
+        <v>0.54139999999999999</v>
+      </c>
+      <c r="AK12" s="1">
+        <v>0.59350000000000003</v>
+      </c>
+      <c r="AL12" s="1">
+        <v>0.55030000000000001</v>
+      </c>
+      <c r="AM12" s="1">
+        <v>0.68530000000000002</v>
+      </c>
+      <c r="AN12" s="1">
+        <v>0.58069999999999999</v>
+      </c>
+      <c r="AO12" s="1">
+        <v>0.84540000000000004</v>
+      </c>
+      <c r="AP12" s="1">
+        <v>0.67659999999999998</v>
+      </c>
+      <c r="AQ12" s="1">
+        <v>0.61319999999999997</v>
+      </c>
+      <c r="AR12" s="1">
+        <v>0.61580000000000001</v>
+      </c>
+      <c r="AS12" s="1">
+        <v>0.75290000000000001</v>
+      </c>
+      <c r="AT12" s="1">
+        <v>0.67879999999999996</v>
+      </c>
+      <c r="AU12" s="1">
+        <v>0.65339999999999998</v>
+      </c>
+      <c r="AV12" s="1">
+        <v>0.65380000000000005</v>
+      </c>
+      <c r="AW12" s="1">
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="AX12" s="1">
+        <v>0.72889999999999999</v>
+      </c>
+      <c r="AY12" s="1">
+        <v>0.68689999999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B13" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I13" s="1">
+        <v>12.1676</v>
+      </c>
+      <c r="J13" s="1">
+        <v>8.8137000000000008</v>
+      </c>
+      <c r="K13" s="1">
+        <v>7.8342000000000001</v>
+      </c>
+      <c r="L13" s="1">
+        <v>6.2252000000000001</v>
+      </c>
+      <c r="M13" s="1">
+        <v>5.8059000000000003</v>
+      </c>
+      <c r="N13" s="1">
+        <v>5.1135000000000002</v>
+      </c>
+      <c r="O13" s="1">
+        <v>4.2605000000000004</v>
+      </c>
+      <c r="P13" s="1">
+        <v>3.3521000000000001</v>
+      </c>
+      <c r="Q13" s="1">
+        <v>3.7713000000000001</v>
+      </c>
+      <c r="R13" s="1">
+        <v>2.9750999999999999</v>
+      </c>
+      <c r="S13" s="1">
+        <v>2.1888000000000001</v>
+      </c>
+      <c r="T13" s="1">
+        <v>1.0874999999999999</v>
+      </c>
+      <c r="U13" s="1">
+        <v>1.9521999999999999</v>
+      </c>
+      <c r="V13" s="1">
+        <v>1.6859999999999999</v>
+      </c>
+      <c r="W13" s="1">
+        <v>1.1573</v>
+      </c>
+      <c r="X13" s="1">
+        <v>2.0760000000000001</v>
+      </c>
+      <c r="Y13" s="1">
+        <v>1.2547999999999999</v>
+      </c>
+      <c r="Z13" s="1">
+        <v>1.9915</v>
+      </c>
+      <c r="AA13" s="1">
+        <v>0.97989999999999999</v>
+      </c>
+      <c r="AB13" s="1">
+        <v>1.5638000000000001</v>
+      </c>
+      <c r="AC13" s="1">
+        <v>0.46820000000000001</v>
+      </c>
+      <c r="AD13" s="1">
+        <v>0.82330000000000003</v>
+      </c>
+      <c r="AE13" s="1">
+        <v>1.2124999999999999</v>
+      </c>
+      <c r="AF13" s="1">
+        <v>1.5492999999999999</v>
+      </c>
+      <c r="AG13" s="1">
+        <v>0.47899999999999998</v>
+      </c>
+      <c r="AH13" s="1">
+        <v>0.54310000000000003</v>
+      </c>
+      <c r="AI13" s="1">
+        <v>0.63149999999999995</v>
+      </c>
+      <c r="AJ13" s="1">
+        <v>0.69889999999999997</v>
+      </c>
+      <c r="AK13" s="1">
+        <v>0.74199999999999999</v>
+      </c>
+      <c r="AL13" s="1">
+        <v>0.76329999999999998</v>
+      </c>
+      <c r="AM13" s="1">
+        <v>0.76770000000000005</v>
+      </c>
+      <c r="AN13" s="1">
+        <v>0.76290000000000002</v>
+      </c>
+      <c r="AO13" s="1">
+        <v>0.76060000000000005</v>
+      </c>
+      <c r="AP13" s="1">
+        <v>0.7762</v>
+      </c>
+      <c r="AQ13" s="1">
+        <v>0.82379999999999998</v>
+      </c>
+      <c r="AR13" s="1">
+        <v>0.90600000000000003</v>
+      </c>
+      <c r="AS13" s="1">
+        <v>1.1672</v>
+      </c>
+      <c r="AT13" s="1">
+        <v>0.95609999999999995</v>
+      </c>
+      <c r="AU13" s="1">
+        <v>0.87660000000000005</v>
+      </c>
+      <c r="AV13" s="1">
+        <v>0.88439999999999996</v>
+      </c>
+      <c r="AW13" s="1">
+        <v>0.94540000000000002</v>
+      </c>
+      <c r="AX13" s="1">
+        <v>0.99639999999999995</v>
+      </c>
+      <c r="AY13" s="1">
+        <v>0.90959999999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B14" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L14" s="1">
+        <v>63.092700000000001</v>
+      </c>
+      <c r="M14" s="1">
+        <v>45.0334</v>
+      </c>
+      <c r="N14" s="1">
+        <v>18.486699999999999</v>
+      </c>
+      <c r="O14" s="1">
+        <v>18.608000000000001</v>
+      </c>
+      <c r="P14" s="1">
+        <v>7.6725000000000003</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>8.3720999999999997</v>
+      </c>
+      <c r="R14" s="1">
+        <v>4.8342999999999998</v>
+      </c>
+      <c r="S14" s="1">
+        <v>4.7374999999999998</v>
+      </c>
+      <c r="T14" s="1">
+        <v>12.7255</v>
+      </c>
+      <c r="U14" s="1">
+        <v>8.7452000000000005</v>
+      </c>
+      <c r="V14" s="1">
+        <v>5.149</v>
+      </c>
+      <c r="W14" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="X14" s="1">
+        <v>2.6092</v>
+      </c>
+      <c r="Y14" s="1">
+        <v>1.653</v>
+      </c>
+      <c r="Z14" s="1">
+        <v>1.8393999999999999</v>
+      </c>
+      <c r="AA14" s="1">
+        <v>2.3845000000000001</v>
+      </c>
+      <c r="AB14" s="1">
+        <v>2.7690000000000001</v>
+      </c>
+      <c r="AC14" s="1">
+        <v>2.883</v>
+      </c>
+      <c r="AD14" s="1">
+        <v>2.7164000000000001</v>
+      </c>
+      <c r="AE14" s="1">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AF14" s="1">
+        <v>1.6960999999999999</v>
+      </c>
+      <c r="AG14" s="1">
+        <v>1.0224</v>
+      </c>
+      <c r="AH14" s="1">
+        <v>5.0904999999999996</v>
+      </c>
+      <c r="AI14" s="1">
+        <v>3.7869000000000002</v>
+      </c>
+      <c r="AJ14" s="1">
+        <v>2.4685000000000001</v>
+      </c>
+      <c r="AK14" s="1">
+        <v>1.339</v>
+      </c>
+      <c r="AL14" s="1">
+        <v>4.4321000000000002</v>
+      </c>
+      <c r="AM14" s="1">
+        <v>2.6738</v>
+      </c>
+      <c r="AN14" s="1">
+        <v>1.4107000000000001</v>
+      </c>
+      <c r="AO14" s="1">
+        <v>3.7309999999999999</v>
+      </c>
+      <c r="AP14" s="1">
+        <v>1.9461999999999999</v>
+      </c>
+      <c r="AQ14" s="1">
+        <v>4.3182999999999998</v>
+      </c>
+      <c r="AR14" s="1">
+        <v>2.2423999999999999</v>
+      </c>
+      <c r="AS14" s="1">
+        <v>1.4419</v>
+      </c>
+      <c r="AT14" s="1">
+        <v>2.2458</v>
+      </c>
+      <c r="AU14" s="1">
+        <v>4.0513000000000003</v>
+      </c>
+      <c r="AV14" s="1">
+        <v>2.0459000000000001</v>
+      </c>
+      <c r="AW14" s="1">
+        <v>3.3957999999999999</v>
+      </c>
+      <c r="AX14" s="1">
+        <v>1.7762</v>
+      </c>
+      <c r="AY14" s="1">
+        <v>2.6551</v>
+      </c>
+    </row>
+    <row r="15" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B15" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="R15" s="1">
+        <v>14.9594</v>
+      </c>
+      <c r="S15" s="1">
+        <v>14.3116</v>
+      </c>
+      <c r="T15" s="1">
+        <v>12.2311</v>
+      </c>
+      <c r="U15" s="1">
+        <v>9.6115999999999993</v>
+      </c>
+      <c r="V15" s="1">
+        <v>33.480800000000002</v>
+      </c>
+      <c r="W15" s="1">
+        <v>27.402899999999999</v>
+      </c>
+      <c r="X15" s="1">
+        <v>21.174399999999999</v>
+      </c>
+      <c r="Y15" s="1">
+        <v>15.769500000000001</v>
+      </c>
+      <c r="Z15" s="1">
+        <v>11.569800000000001</v>
+      </c>
+      <c r="AA15" s="1">
+        <v>8.5905000000000005</v>
+      </c>
+      <c r="AB15" s="1">
+        <v>5.4943999999999997</v>
+      </c>
+      <c r="AC15" s="1">
+        <v>3.1288</v>
+      </c>
+      <c r="AD15" s="1">
+        <v>2.347</v>
+      </c>
+      <c r="AE15" s="1">
+        <v>3.0129000000000001</v>
+      </c>
+      <c r="AF15" s="1">
+        <v>2.9232999999999998</v>
+      </c>
+      <c r="AG15" s="1">
+        <v>1.8461000000000001</v>
+      </c>
+      <c r="AH15" s="1">
+        <v>6.1643999999999997</v>
+      </c>
+      <c r="AI15" s="1">
+        <v>3.1227</v>
+      </c>
+      <c r="AJ15" s="1">
+        <v>7.9588999999999999</v>
+      </c>
+      <c r="AK15" s="1">
+        <v>3.6326999999999998</v>
+      </c>
+      <c r="AL15" s="1">
+        <v>7.9225000000000003</v>
+      </c>
+      <c r="AM15" s="1">
+        <v>3.3125</v>
+      </c>
+      <c r="AN15" s="1">
+        <v>6.3601000000000001</v>
+      </c>
+      <c r="AO15" s="1">
+        <v>10.616300000000001</v>
+      </c>
+      <c r="AP15" s="1">
+        <v>4.2582000000000004</v>
+      </c>
+      <c r="AQ15" s="1">
+        <v>6.9177999999999997</v>
+      </c>
+      <c r="AR15" s="1">
+        <v>10.2485</v>
+      </c>
+      <c r="AS15" s="1">
+        <v>3.8751000000000002</v>
+      </c>
+      <c r="AT15" s="1">
+        <v>5.3685</v>
+      </c>
+      <c r="AU15" s="1">
+        <v>7.3761999999999999</v>
+      </c>
+      <c r="AV15" s="1">
+        <v>9.6674000000000007</v>
+      </c>
+      <c r="AW15" s="1">
+        <v>12.0786</v>
+      </c>
+      <c r="AX15" s="1">
+        <v>4.2385999999999999</v>
+      </c>
+      <c r="AY15" s="1">
+        <v>5.0271999999999997</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C3:AY15">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="10"/>
+        <cfvo type="max"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F192E7DF-432D-405C-9CC1-E8A78B1D27F2}">
+  <dimension ref="B1:AY20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="51" width="5.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:51" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="K2" s="1">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M2" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="N2" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="O2" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="P2" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="R2" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="S2" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="T2" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="U2" s="1">
+        <v>2</v>
+      </c>
+      <c r="V2" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="W2" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="X2" s="1">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>2.4</v>
+      </c>
+      <c r="Z2" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="AA2" s="1">
+        <v>2.6</v>
+      </c>
+      <c r="AB2" s="1">
+        <v>2.7</v>
+      </c>
+      <c r="AC2" s="1">
+        <v>2.8</v>
+      </c>
+      <c r="AD2" s="1">
+        <v>2.9</v>
+      </c>
+      <c r="AE2" s="1">
+        <v>3</v>
+      </c>
+      <c r="AF2" s="1">
+        <v>3.1</v>
+      </c>
+      <c r="AG2" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="AH2" s="1">
+        <v>3.3</v>
+      </c>
+      <c r="AI2" s="1">
+        <v>3.4</v>
+      </c>
+      <c r="AJ2" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="AK2" s="1">
+        <v>3.6</v>
+      </c>
+      <c r="AL2" s="1">
+        <v>3.7</v>
+      </c>
+      <c r="AM2" s="1">
+        <v>3.8</v>
+      </c>
+      <c r="AN2" s="1">
+        <v>3.9</v>
+      </c>
+      <c r="AO2" s="1">
+        <v>4</v>
+      </c>
+      <c r="AP2" s="1">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AQ2" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="AR2" s="1">
+        <v>4.3</v>
+      </c>
+      <c r="AS2" s="1">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AT2" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="AU2" s="1">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AV2" s="1">
+        <v>4.7</v>
+      </c>
+      <c r="AW2" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="AX2" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="AY2" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B3" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.41610000000000003</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.11559999999999999</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.2923</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.1144</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0.12039999999999999</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0.1719</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0.15890000000000001</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0.1792</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0.17929999999999999</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0.23169999999999999</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0.26669999999999999</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0.32169999999999999</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0.44</v>
+      </c>
+      <c r="P3" s="1">
+        <v>0.40039999999999998</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AG3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AL3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AM3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AN3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AO3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AP3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AQ3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AR3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AS3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AT3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AU3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AV3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AW3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AX3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AY3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B4" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.59670000000000001</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5.11E-2</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1">
+        <v>4.7E-2</v>
+      </c>
+      <c r="G4" s="1">
+        <v>7.6300000000000007E-2</v>
+      </c>
+      <c r="H4" s="1">
+        <v>7.2300000000000003E-2</v>
+      </c>
+      <c r="I4" s="1">
+        <v>8.3299999999999999E-2</v>
+      </c>
+      <c r="J4" s="1">
+        <v>9.5100000000000004E-2</v>
+      </c>
+      <c r="K4" s="1">
+        <v>8.9899999999999994E-2</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0.17249999999999999</v>
+      </c>
+      <c r="M4" s="1">
+        <v>9.9099999999999994E-2</v>
+      </c>
+      <c r="N4" s="1">
+        <v>0.1168</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0.16339999999999999</v>
+      </c>
+      <c r="P4" s="1">
+        <v>0.15479999999999999</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>0.1258</v>
+      </c>
+      <c r="R4" s="1">
+        <v>0.25340000000000001</v>
+      </c>
+      <c r="S4" s="1">
+        <v>0.47199999999999998</v>
+      </c>
+      <c r="T4" s="1">
+        <v>0.16370000000000001</v>
+      </c>
+      <c r="U4" s="1">
+        <v>0.2223</v>
+      </c>
+      <c r="V4" s="1">
+        <v>0.24360000000000001</v>
+      </c>
+      <c r="W4" s="1">
+        <v>0.23719999999999999</v>
+      </c>
+      <c r="X4" s="1">
+        <v>0.25219999999999998</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>0.27900000000000003</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>0.2064</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AB4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AG4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AH4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AK4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AL4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AM4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AN4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AO4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AP4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AQ4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AR4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AS4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AT4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AU4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AV4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AW4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AX4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AY4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B5" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1.8207</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1.1791</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.26729999999999998</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.78559999999999997</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0.58189999999999997</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3.04E-2</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0.1696</v>
+      </c>
+      <c r="J5" s="1">
+        <v>4.3499999999999997E-2</v>
+      </c>
+      <c r="K5" s="1">
+        <v>4.7399999999999998E-2</v>
+      </c>
+      <c r="L5" s="1">
+        <v>4.3700000000000003E-2</v>
+      </c>
+      <c r="M5" s="1">
+        <v>4.87E-2</v>
+      </c>
+      <c r="N5" s="1">
+        <v>0.4173</v>
+      </c>
+      <c r="O5" s="1">
+        <v>0.10489999999999999</v>
+      </c>
+      <c r="P5" s="1">
+        <v>0.1308</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>0.1522</v>
+      </c>
+      <c r="R5" s="1">
+        <v>8.1100000000000005E-2</v>
+      </c>
+      <c r="S5" s="1">
+        <v>9.4299999999999995E-2</v>
+      </c>
+      <c r="T5" s="1">
+        <v>0.2671</v>
+      </c>
+      <c r="U5" s="1">
+        <v>0.24640000000000001</v>
+      </c>
+      <c r="V5" s="1">
+        <v>0.18210000000000001</v>
+      </c>
+      <c r="W5" s="1">
+        <v>0.19539999999999999</v>
+      </c>
+      <c r="X5" s="1">
+        <v>0.1041</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>0.30940000000000001</v>
+      </c>
+      <c r="Z5" s="1">
+        <v>0.124</v>
+      </c>
+      <c r="AA5" s="1">
+        <v>0.1285</v>
+      </c>
+      <c r="AB5" s="1">
+        <v>0.36449999999999999</v>
+      </c>
+      <c r="AC5" s="1">
+        <v>0.31759999999999999</v>
+      </c>
+      <c r="AD5" s="1">
+        <v>0.1986</v>
+      </c>
+      <c r="AE5" s="1">
+        <v>1.0629</v>
+      </c>
+      <c r="AF5" s="1">
+        <v>0.15060000000000001</v>
+      </c>
+      <c r="AG5" s="1">
+        <v>0.63370000000000004</v>
+      </c>
+      <c r="AH5" s="1">
+        <v>0.36199999999999999</v>
+      </c>
+      <c r="AI5" s="1">
+        <v>1.14E-2</v>
+      </c>
+      <c r="AJ5" s="1">
+        <v>0.94020000000000004</v>
+      </c>
+      <c r="AK5" s="1">
+        <v>0.83409999999999995</v>
+      </c>
+      <c r="AL5" s="1">
+        <v>0.215</v>
+      </c>
+      <c r="AM5" s="1">
+        <v>0.187</v>
+      </c>
+      <c r="AN5" s="1">
+        <v>0.21260000000000001</v>
+      </c>
+      <c r="AO5" s="1">
+        <v>0.86419999999999997</v>
+      </c>
+      <c r="AP5" s="1">
+        <v>0.34670000000000001</v>
+      </c>
+      <c r="AQ5" s="1">
+        <v>0.25929999999999997</v>
+      </c>
+      <c r="AR5" s="28">
+        <v>5.5511E-17</v>
+      </c>
+      <c r="AS5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AT5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AU5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AV5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AW5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AX5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AY5" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B6" s="1">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2.7145000000000001</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1.1274999999999999</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.21510000000000001</v>
+      </c>
+      <c r="G6" s="1">
+        <v>3.8800000000000001E-2</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1.4342999999999999</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1.9699999999999999E-2</v>
+      </c>
+      <c r="J6" s="1">
+        <v>3.1E-2</v>
+      </c>
+      <c r="K6" s="1">
+        <v>9.1800000000000007E-2</v>
+      </c>
+      <c r="L6" s="1">
+        <v>9.1999999999999998E-3</v>
+      </c>
+      <c r="M6" s="1">
+        <v>1.5100000000000001E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>5.11E-2</v>
+      </c>
+      <c r="O6" s="1">
+        <v>4.6399999999999997E-2</v>
+      </c>
+      <c r="P6" s="1">
+        <v>2.2800000000000001E-2</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>0.2198</v>
+      </c>
+      <c r="R6" s="1">
+        <v>2.9399999999999999E-2</v>
+      </c>
+      <c r="S6" s="1">
+        <v>0.34899999999999998</v>
+      </c>
+      <c r="T6" s="1">
+        <v>0.1923</v>
+      </c>
+      <c r="U6" s="1">
+        <v>0.14729999999999999</v>
+      </c>
+      <c r="V6" s="1">
+        <v>0.2253</v>
+      </c>
+      <c r="W6" s="28">
+        <v>5476.3</v>
+      </c>
+      <c r="X6" s="1">
+        <v>0.14729999999999999</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>9.0700000000000003E-2</v>
+      </c>
+      <c r="Z6" s="1">
+        <v>6.6400000000000001E-2</v>
+      </c>
+      <c r="AA6" s="1">
+        <v>0.21729999999999999</v>
+      </c>
+      <c r="AB6" s="1">
+        <v>0.90790000000000004</v>
+      </c>
+      <c r="AC6" s="1">
+        <v>0.72219999999999995</v>
+      </c>
+      <c r="AD6" s="1">
+        <v>0.91349999999999998</v>
+      </c>
+      <c r="AE6" s="1">
+        <v>0.85070000000000001</v>
+      </c>
+      <c r="AF6" s="1">
+        <v>0.84530000000000005</v>
+      </c>
+      <c r="AG6" s="1">
+        <v>0.2452</v>
+      </c>
+      <c r="AH6" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="AI6" s="1">
+        <v>0.51759999999999995</v>
+      </c>
+      <c r="AJ6" s="1">
+        <v>9.06E-2</v>
+      </c>
+      <c r="AK6" s="1">
+        <v>0.1358</v>
+      </c>
+      <c r="AL6" s="1">
+        <v>0.79059999999999997</v>
+      </c>
+      <c r="AM6" s="1">
+        <v>0.48</v>
+      </c>
+      <c r="AN6" s="1">
+        <v>0.58889999999999998</v>
+      </c>
+      <c r="AO6" s="1">
+        <v>0.4824</v>
+      </c>
+      <c r="AP6" s="1">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="AQ6" s="1">
+        <v>0.71140000000000003</v>
+      </c>
+      <c r="AR6" s="1">
+        <v>0.57050000000000001</v>
+      </c>
+      <c r="AS6" s="1">
+        <v>0.47410000000000002</v>
+      </c>
+      <c r="AT6" s="1">
+        <v>0.2331</v>
+      </c>
+      <c r="AU6" s="28">
+        <v>1.3718000000000001E-8</v>
+      </c>
+      <c r="AV6" s="1">
+        <v>0.19109999999999999</v>
+      </c>
+      <c r="AW6" s="1">
+        <v>0.58150000000000002</v>
+      </c>
+      <c r="AX6" s="1">
+        <v>0.5353</v>
+      </c>
+      <c r="AY6" s="1">
+        <v>0.3715</v>
+      </c>
+    </row>
+    <row r="7" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B7" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C7" s="1">
+        <v>4.0782999999999996</v>
+      </c>
+      <c r="D7" s="1">
+        <v>3.2130000000000001</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.105</v>
+      </c>
+      <c r="F7" s="1">
+        <v>2.3033999999999999</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0.89649999999999996</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0.56699999999999995</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.39600000000000002</v>
+      </c>
+      <c r="J7" s="1">
+        <v>2.4318</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0.1091</v>
+      </c>
+      <c r="L7" s="1">
+        <v>0.42430000000000001</v>
+      </c>
+      <c r="M7" s="28">
+        <v>5.9971999999999999E-13</v>
+      </c>
+      <c r="N7" s="28">
+        <v>4.9631000000000002E-14</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="28">
+        <v>3.6123999999999998E-12</v>
+      </c>
+      <c r="R7" s="1">
+        <v>0.87819999999999998</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="W7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="X7" s="1">
+        <v>0.1087</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="28">
+        <v>1.1102000000000001E-18</v>
+      </c>
+      <c r="AA7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC7" s="28">
+        <v>2.7089E-16</v>
+      </c>
+      <c r="AD7" s="1">
+        <v>0.76749999999999996</v>
+      </c>
+      <c r="AE7" s="1">
+        <v>0.24709999999999999</v>
+      </c>
+      <c r="AF7" s="1">
+        <v>0.58340000000000003</v>
+      </c>
+      <c r="AG7" s="1">
+        <v>0.62219999999999998</v>
+      </c>
+      <c r="AH7" s="1">
+        <v>0.1656</v>
+      </c>
+      <c r="AI7" s="1">
+        <v>0.6714</v>
+      </c>
+      <c r="AJ7" s="1">
+        <v>0.47039999999999998</v>
+      </c>
+      <c r="AK7" s="1">
+        <v>0.1978</v>
+      </c>
+      <c r="AL7" s="1">
+        <v>0.46879999999999999</v>
+      </c>
+      <c r="AM7" s="1">
+        <v>0.57530000000000003</v>
+      </c>
+      <c r="AN7" s="1">
+        <v>0.2429</v>
+      </c>
+      <c r="AO7" s="1">
+        <v>0.30740000000000001</v>
+      </c>
+      <c r="AP7" s="1">
+        <v>0.2127</v>
+      </c>
+      <c r="AQ7" s="1">
+        <v>0.4657</v>
+      </c>
+      <c r="AR7" s="1">
+        <v>0.41370000000000001</v>
+      </c>
+      <c r="AS7" s="1">
+        <v>0.21440000000000001</v>
+      </c>
+      <c r="AT7" s="1">
+        <v>0.21010000000000001</v>
+      </c>
+      <c r="AU7" s="1">
+        <v>5.5999999999999999E-3</v>
+      </c>
+      <c r="AV7" s="1">
+        <v>1.3754</v>
+      </c>
+      <c r="AW7" s="1">
+        <v>0.43280000000000002</v>
+      </c>
+      <c r="AX7" s="1">
+        <v>0.4143</v>
+      </c>
+      <c r="AY7" s="1">
+        <v>0.28510000000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B8" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.1888</v>
+      </c>
+      <c r="D8" s="1">
+        <v>3.9087999999999998</v>
+      </c>
+      <c r="E8" s="1">
+        <v>2.9902000000000002</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1.4116</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1.9235</v>
+      </c>
+      <c r="H8" s="1">
+        <v>1.6049</v>
+      </c>
+      <c r="I8" s="1">
+        <v>1.194</v>
+      </c>
+      <c r="J8" s="1">
+        <v>1.1792</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0.27139999999999997</v>
+      </c>
+      <c r="L8" s="1">
+        <v>0.36930000000000002</v>
+      </c>
+      <c r="M8" s="1">
+        <v>0.86760000000000004</v>
+      </c>
+      <c r="N8" s="28">
+        <v>2.8721999999999998E-12</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P8" s="1">
+        <v>0.1908</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>2.621</v>
+      </c>
+      <c r="R8" s="1">
+        <v>1.4684999999999999</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T8" s="1">
+        <v>0.36630000000000001</v>
+      </c>
+      <c r="U8" s="1">
+        <v>0.17019999999999999</v>
+      </c>
+      <c r="V8" s="1">
+        <v>0.55969999999999998</v>
+      </c>
+      <c r="W8" s="1">
+        <v>0.23630000000000001</v>
+      </c>
+      <c r="X8" s="1">
+        <v>0.24560000000000001</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>0.22550000000000001</v>
+      </c>
+      <c r="Z8" s="1">
+        <v>0.28670000000000001</v>
+      </c>
+      <c r="AA8" s="1">
+        <v>0.22159999999999999</v>
+      </c>
+      <c r="AB8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC8" s="1">
+        <v>0.35460000000000003</v>
+      </c>
+      <c r="AD8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE8" s="1">
+        <v>0.63539999999999996</v>
+      </c>
+      <c r="AF8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AG8" s="1">
+        <v>0.43190000000000001</v>
+      </c>
+      <c r="AH8" s="1">
+        <v>4.3151000000000002</v>
+      </c>
+      <c r="AI8" s="1">
+        <v>0.56040000000000001</v>
+      </c>
+      <c r="AJ8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AK8" s="1">
+        <v>0.40939999999999999</v>
+      </c>
+      <c r="AL8" s="1">
+        <v>3.2928999999999999</v>
+      </c>
+      <c r="AM8" s="1">
+        <v>0.5202</v>
+      </c>
+      <c r="AN8" s="1">
+        <v>6.4207000000000001</v>
+      </c>
+      <c r="AO8" s="1">
+        <v>0.64510000000000001</v>
+      </c>
+      <c r="AP8" s="1">
+        <v>1.4396</v>
+      </c>
+      <c r="AQ8" s="1">
+        <v>0.52339999999999998</v>
+      </c>
+      <c r="AR8" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="AS8" s="1">
+        <v>0.53</v>
+      </c>
+      <c r="AT8" s="1">
+        <v>0.58220000000000005</v>
+      </c>
+      <c r="AU8" s="1">
+        <v>0.6079</v>
+      </c>
+      <c r="AV8" s="1">
+        <v>0.82430000000000003</v>
+      </c>
+      <c r="AW8" s="1">
+        <v>0.68240000000000001</v>
+      </c>
+      <c r="AX8" s="1">
+        <v>0.97860000000000003</v>
+      </c>
+      <c r="AY8" s="1">
+        <v>0.73360000000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B9" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="1">
+        <v>3.8849999999999998</v>
+      </c>
+      <c r="E9" s="1">
+        <v>6.2121000000000004</v>
+      </c>
+      <c r="F9" s="1">
+        <v>3.3452000000000002</v>
+      </c>
+      <c r="G9" s="1">
+        <v>4.7830000000000004</v>
+      </c>
+      <c r="H9" s="1">
+        <v>1.3882000000000001</v>
+      </c>
+      <c r="I9" s="1">
+        <v>1.6618999999999999</v>
+      </c>
+      <c r="J9" s="1">
+        <v>2.1051000000000002</v>
+      </c>
+      <c r="K9" s="1">
+        <v>1.0148999999999999</v>
+      </c>
+      <c r="L9" s="1">
+        <v>0.62109999999999999</v>
+      </c>
+      <c r="M9" s="1">
+        <v>1.6282000000000001</v>
+      </c>
+      <c r="N9" s="1">
+        <v>0.2452</v>
+      </c>
+      <c r="O9" s="1">
+        <v>0.28810000000000002</v>
+      </c>
+      <c r="P9" s="1">
+        <v>0.42299999999999999</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>0.60409999999999997</v>
+      </c>
+      <c r="R9" s="1">
+        <v>2.7989999999999999</v>
+      </c>
+      <c r="S9" s="1">
+        <v>0.54090000000000005</v>
+      </c>
+      <c r="T9" s="1">
+        <v>0.87319999999999998</v>
+      </c>
+      <c r="U9" s="1">
+        <v>0.39510000000000001</v>
+      </c>
+      <c r="V9" s="1">
+        <v>0.36430000000000001</v>
+      </c>
+      <c r="W9" s="1">
+        <v>0.38490000000000002</v>
+      </c>
+      <c r="X9" s="1">
+        <v>0.50229999999999997</v>
+      </c>
+      <c r="Y9" s="1">
+        <v>0.44579999999999997</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA9" s="1">
+        <v>0.32100000000000001</v>
+      </c>
+      <c r="AB9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC9" s="1">
+        <v>0.84340000000000004</v>
+      </c>
+      <c r="AD9" s="1">
+        <v>0.39150000000000001</v>
+      </c>
+      <c r="AE9" s="1">
+        <v>2.0506000000000002</v>
+      </c>
+      <c r="AF9" s="1">
+        <v>4.1798999999999999</v>
+      </c>
+      <c r="AG9" s="28">
+        <v>7.5494999999999995E-17</v>
+      </c>
+      <c r="AH9" s="1">
+        <v>0.5252</v>
+      </c>
+      <c r="AI9" s="1">
+        <v>0.88739999999999997</v>
+      </c>
+      <c r="AJ9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AK9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AL9" s="28">
+        <v>1.6954000000000001E-8</v>
+      </c>
+      <c r="AM9" s="1">
+        <v>0.56930000000000003</v>
+      </c>
+      <c r="AN9" s="1">
+        <v>1.0162</v>
+      </c>
+      <c r="AO9" s="28">
+        <v>6.2172000000000005E-17</v>
+      </c>
+      <c r="AP9" s="1">
+        <v>0.94279999999999997</v>
+      </c>
+      <c r="AQ9" s="1">
+        <v>1.1197999999999999</v>
+      </c>
+      <c r="AR9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AS9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AT9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AU9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AV9" s="1">
+        <v>1.0342</v>
+      </c>
+      <c r="AW9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AX9" s="28">
+        <v>1.6679999999999999E-4</v>
+      </c>
+      <c r="AY9" s="1">
+        <v>1.7331000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B10" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="1">
+        <v>6.5934999999999997</v>
+      </c>
+      <c r="F10" s="1">
+        <v>3.9708999999999999</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.7565</v>
+      </c>
+      <c r="H10" s="1">
+        <v>2.1267</v>
+      </c>
+      <c r="I10" s="1">
+        <v>1.8552999999999999</v>
+      </c>
+      <c r="J10" s="1">
+        <v>1.9495</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0.94169999999999998</v>
+      </c>
+      <c r="L10" s="1">
+        <v>0.85440000000000005</v>
+      </c>
+      <c r="M10" s="1">
+        <v>1.4011</v>
+      </c>
+      <c r="N10" s="1">
+        <v>1.8972</v>
+      </c>
+      <c r="O10" s="1">
+        <v>1.9249000000000001</v>
+      </c>
+      <c r="P10" s="1">
+        <v>0.34010000000000001</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>0.57469999999999999</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S10" s="1">
+        <v>0.48849999999999999</v>
+      </c>
+      <c r="T10" s="28">
+        <v>4.9569999999999997E-14</v>
+      </c>
+      <c r="U10" s="1">
+        <v>0.88549999999999995</v>
+      </c>
+      <c r="V10" s="1">
+        <v>1.1872</v>
+      </c>
+      <c r="W10" s="1">
+        <v>1.9753000000000001</v>
+      </c>
+      <c r="X10" s="1">
+        <v>1.1806000000000001</v>
+      </c>
+      <c r="Y10" s="1">
+        <v>0.66149999999999998</v>
+      </c>
+      <c r="Z10" s="1">
+        <v>2.3E-3</v>
+      </c>
+      <c r="AA10" s="1">
+        <v>0.73970000000000002</v>
+      </c>
+      <c r="AB10" s="1">
+        <v>0.74370000000000003</v>
+      </c>
+      <c r="AC10" s="1">
+        <v>0.70089999999999997</v>
+      </c>
+      <c r="AD10" s="1">
+        <v>2.9554</v>
+      </c>
+      <c r="AE10" s="1">
+        <v>1.5248999999999999</v>
+      </c>
+      <c r="AF10" s="1">
+        <v>0.68279999999999996</v>
+      </c>
+      <c r="AG10" s="1">
+        <v>0.39810000000000001</v>
+      </c>
+      <c r="AH10" s="1">
+        <v>1.9433</v>
+      </c>
+      <c r="AI10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ10" s="1">
+        <v>0.95089999999999997</v>
+      </c>
+      <c r="AK10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AL10" s="1">
+        <v>1.7458</v>
+      </c>
+      <c r="AM10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AN10" s="1">
+        <v>0.27800000000000002</v>
+      </c>
+      <c r="AO10" s="1">
+        <v>1.2222999999999999</v>
+      </c>
+      <c r="AP10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AQ10" s="1">
+        <v>1.4177</v>
+      </c>
+      <c r="AR10" s="1">
+        <v>1.2301</v>
+      </c>
+      <c r="AS10" s="1">
+        <v>0.93810000000000004</v>
+      </c>
+      <c r="AT10" s="1">
+        <v>0.90229999999999999</v>
+      </c>
+      <c r="AU10" s="28">
+        <v>4.6494E-12</v>
+      </c>
+      <c r="AV10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AW10" s="1">
+        <v>2.3016000000000001</v>
+      </c>
+      <c r="AX10" s="1">
+        <v>1.1776</v>
+      </c>
+      <c r="AY10" s="1">
+        <v>0.63449999999999995</v>
+      </c>
+    </row>
+    <row r="11" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B11" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="28">
+        <v>5.7084000000000001</v>
+      </c>
+      <c r="G11" s="1">
+        <v>3.5228000000000002</v>
+      </c>
+      <c r="H11" s="1">
+        <v>3.4794</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0.53779999999999994</v>
+      </c>
+      <c r="J11" s="1">
+        <v>2.8347000000000002</v>
+      </c>
+      <c r="K11" s="1">
+        <v>2.6903000000000001</v>
+      </c>
+      <c r="L11" s="1">
+        <v>4.7827999999999999</v>
+      </c>
+      <c r="M11" s="1">
+        <v>2.387</v>
+      </c>
+      <c r="N11" s="1">
+        <v>1.1605000000000001</v>
+      </c>
+      <c r="O11" s="1">
+        <v>1.9159999999999999</v>
+      </c>
+      <c r="P11" s="1">
+        <v>1.4534</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>2.6374</v>
+      </c>
+      <c r="R11" s="1">
+        <v>1.0477000000000001</v>
+      </c>
+      <c r="S11" s="1">
+        <v>0.75649999999999995</v>
+      </c>
+      <c r="T11" s="1">
+        <v>0.86670000000000003</v>
+      </c>
+      <c r="U11" s="1">
+        <v>1.5668</v>
+      </c>
+      <c r="V11" s="28">
+        <v>3.2862999999999998E-16</v>
+      </c>
+      <c r="W11" s="1">
+        <v>2.6602999999999999</v>
+      </c>
+      <c r="X11" s="1">
+        <v>1.7577</v>
+      </c>
+      <c r="Y11" s="1">
+        <v>0.55930000000000002</v>
+      </c>
+      <c r="Z11" s="1">
+        <v>0.98450000000000004</v>
+      </c>
+      <c r="AA11" s="1">
+        <v>0.62560000000000004</v>
+      </c>
+      <c r="AB11" s="1">
+        <v>1.1798999999999999</v>
+      </c>
+      <c r="AC11" s="1">
+        <v>0.89459999999999995</v>
+      </c>
+      <c r="AD11" s="1">
+        <v>0.82179999999999997</v>
+      </c>
+      <c r="AE11" s="1">
+        <v>0.8911</v>
+      </c>
+      <c r="AF11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AG11" s="1">
+        <v>0.78390000000000004</v>
+      </c>
+      <c r="AH11" s="1">
+        <v>0.97309999999999997</v>
+      </c>
+      <c r="AI11" s="1">
+        <v>0.50029999999999997</v>
+      </c>
+      <c r="AJ11" s="1">
+        <v>1.0402</v>
+      </c>
+      <c r="AK11" s="1">
+        <v>1.0073000000000001</v>
+      </c>
+      <c r="AL11" s="1">
+        <v>4.8658999999999999</v>
+      </c>
+      <c r="AM11" s="28">
+        <v>7.2440000000000002E-13</v>
+      </c>
+      <c r="AN11" s="1">
+        <v>4.0883000000000003</v>
+      </c>
+      <c r="AO11" s="1">
+        <v>5.91E-2</v>
+      </c>
+      <c r="AP11" s="1">
+        <v>1.1760999999999999</v>
+      </c>
+      <c r="AQ11" s="1">
+        <v>3.1154999999999999</v>
+      </c>
+      <c r="AR11" s="1">
+        <v>3.1511999999999998</v>
+      </c>
+      <c r="AS11" s="1">
+        <v>6.2747000000000002</v>
+      </c>
+      <c r="AT11" s="28">
+        <v>4.9342000000000001E-14</v>
+      </c>
+      <c r="AU11" s="1">
+        <v>5.1928000000000001</v>
+      </c>
+      <c r="AV11" s="1">
+        <v>0.55900000000000005</v>
+      </c>
+      <c r="AW11" s="1">
+        <v>2.0621</v>
+      </c>
+      <c r="AX11" s="1">
+        <v>1.0154000000000001</v>
+      </c>
+      <c r="AY11" s="28">
+        <v>9.8405999999999995E-14</v>
+      </c>
+    </row>
+    <row r="12" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B12" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="28">
+        <v>2.2482000000000002</v>
+      </c>
+      <c r="H12" s="28">
+        <v>3.8944000000000001</v>
+      </c>
+      <c r="I12" s="1">
+        <v>5.2839</v>
+      </c>
+      <c r="J12" s="1">
+        <v>2.1116999999999999</v>
+      </c>
+      <c r="K12" s="1">
+        <v>3.6751</v>
+      </c>
+      <c r="L12" s="1">
+        <v>2.8553999999999999</v>
+      </c>
+      <c r="M12" s="1">
+        <v>2.7161</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1.5026999999999999</v>
+      </c>
+      <c r="O12" s="1">
+        <v>2.8572000000000002</v>
+      </c>
+      <c r="P12" s="1">
+        <v>4.8402000000000003</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>6.2297000000000002</v>
+      </c>
+      <c r="R12" s="1">
+        <v>4.9635999999999996</v>
+      </c>
+      <c r="S12" s="28">
+        <v>9.9256999999999996E-14</v>
+      </c>
+      <c r="T12" s="1">
+        <v>0.6482</v>
+      </c>
+      <c r="U12" s="1">
+        <v>1.5059</v>
+      </c>
+      <c r="V12" s="1">
+        <v>5.9149000000000003</v>
+      </c>
+      <c r="W12" s="1">
+        <v>3.4169999999999998</v>
+      </c>
+      <c r="X12" s="1">
+        <v>2.2343000000000002</v>
+      </c>
+      <c r="Y12" s="1">
+        <v>0.69650000000000001</v>
+      </c>
+      <c r="Z12" s="1">
+        <v>1.3874</v>
+      </c>
+      <c r="AA12" s="28">
+        <v>1.8679999999999999E-4</v>
+      </c>
+      <c r="AB12" s="1">
+        <v>0.94389999999999996</v>
+      </c>
+      <c r="AC12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AD12" s="1">
+        <v>1.9322999999999999</v>
+      </c>
+      <c r="AE12" s="1">
+        <v>1.3861000000000001</v>
+      </c>
+      <c r="AF12" s="1">
+        <v>1.7461</v>
+      </c>
+      <c r="AG12" s="1">
+        <v>1.5733999999999999</v>
+      </c>
+      <c r="AH12" s="1">
+        <v>0.69299999999999995</v>
+      </c>
+      <c r="AI12" s="1">
+        <v>8.4276999999999997</v>
+      </c>
+      <c r="AJ12" s="1">
+        <v>2E-3</v>
+      </c>
+      <c r="AK12" s="1">
+        <v>1.9380999999999999</v>
+      </c>
+      <c r="AL12" s="1">
+        <v>2.1078999999999999</v>
+      </c>
+      <c r="AM12" s="1">
+        <v>2.1017999999999999</v>
+      </c>
+      <c r="AN12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AO12" s="1">
+        <v>13.4237</v>
+      </c>
+      <c r="AP12" s="1">
+        <v>2.5270999999999999</v>
+      </c>
+      <c r="AQ12" s="1">
+        <v>1.2738</v>
+      </c>
+      <c r="AR12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AS12" s="28">
+        <v>1.0658E-16</v>
+      </c>
+      <c r="AT12" s="1">
+        <v>2.3751000000000002</v>
+      </c>
+      <c r="AU12" s="1">
+        <v>10.742900000000001</v>
+      </c>
+      <c r="AV12" s="1">
+        <v>1.3691</v>
+      </c>
+      <c r="AW12" s="28">
+        <v>1.5084E-5</v>
+      </c>
+      <c r="AX12" s="1">
+        <v>4.9781000000000004</v>
+      </c>
+      <c r="AY12" s="1">
+        <v>4.2257999999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B13" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I13" s="1">
+        <v>14.4291</v>
+      </c>
+      <c r="J13" s="1">
+        <v>6.1852</v>
+      </c>
+      <c r="K13" s="1">
+        <v>10.341200000000001</v>
+      </c>
+      <c r="L13" s="1">
+        <v>4.7329999999999997</v>
+      </c>
+      <c r="M13" s="1">
+        <v>2.1503999999999999</v>
+      </c>
+      <c r="N13" s="1">
+        <v>2.9497</v>
+      </c>
+      <c r="O13" s="1">
+        <v>4.4478</v>
+      </c>
+      <c r="P13" s="1">
+        <v>2.8793000000000002</v>
+      </c>
+      <c r="Q13" s="1">
+        <v>9.6168999999999993</v>
+      </c>
+      <c r="R13" s="1">
+        <v>3.8395000000000001</v>
+      </c>
+      <c r="S13" s="1">
+        <v>1.7901</v>
+      </c>
+      <c r="T13" s="1">
+        <v>3.8222</v>
+      </c>
+      <c r="U13" s="1">
+        <v>24.678899999999999</v>
+      </c>
+      <c r="V13" s="1">
+        <v>2.7585999999999999</v>
+      </c>
+      <c r="W13" s="1">
+        <v>13.604699999999999</v>
+      </c>
+      <c r="X13" s="1">
+        <v>2.6004</v>
+      </c>
+      <c r="Y13" s="1">
+        <v>2.48</v>
+      </c>
+      <c r="Z13" s="1">
+        <v>0.22359999999999999</v>
+      </c>
+      <c r="AA13" s="1">
+        <v>2.1991999999999998</v>
+      </c>
+      <c r="AB13" s="1">
+        <v>0.39579999999999999</v>
+      </c>
+      <c r="AC13" s="1">
+        <v>6.2619999999999996</v>
+      </c>
+      <c r="AD13" s="1">
+        <v>13.936999999999999</v>
+      </c>
+      <c r="AE13" s="1">
+        <v>0.90180000000000005</v>
+      </c>
+      <c r="AF13" s="1">
+        <v>0.95750000000000002</v>
+      </c>
+      <c r="AG13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AH13" s="1">
+        <v>0.51080000000000003</v>
+      </c>
+      <c r="AI13" s="28">
+        <v>6.6130999999999996E-10</v>
+      </c>
+      <c r="AJ13" s="28">
+        <v>3.8858E-16</v>
+      </c>
+      <c r="AK13" s="1">
+        <v>15.8522</v>
+      </c>
+      <c r="AL13" s="1">
+        <v>5.8545999999999996</v>
+      </c>
+      <c r="AM13" s="1">
+        <v>2.9828000000000001</v>
+      </c>
+      <c r="AN13" s="1">
+        <v>38.828699999999998</v>
+      </c>
+      <c r="AO13" s="1">
+        <v>1.0666</v>
+      </c>
+      <c r="AP13" s="1">
+        <v>0.66869999999999996</v>
+      </c>
+      <c r="AQ13" s="1">
+        <v>1.1839</v>
+      </c>
+      <c r="AR13" s="1">
+        <v>1.2215</v>
+      </c>
+      <c r="AS13" s="1">
+        <v>13.1357</v>
+      </c>
+      <c r="AT13" s="1">
+        <v>34.671199999999999</v>
+      </c>
+      <c r="AU13" s="1">
+        <v>6.2782</v>
+      </c>
+      <c r="AV13" s="28">
+        <v>9.9183000000000003E-14</v>
+      </c>
+      <c r="AW13" s="28">
+        <v>6.3061000000000001E-16</v>
+      </c>
+      <c r="AX13" s="1">
+        <v>21.1496</v>
+      </c>
+      <c r="AY13" s="1">
+        <v>1.4510000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B14" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L14" s="1">
+        <v>14.7263</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0.48359999999999997</v>
+      </c>
+      <c r="N14" s="1">
+        <v>11.6005</v>
+      </c>
+      <c r="O14" s="1">
+        <v>15.3027</v>
+      </c>
+      <c r="P14" s="1">
+        <v>43.913400000000003</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>14.9612</v>
+      </c>
+      <c r="R14" s="1">
+        <v>4.6788999999999996</v>
+      </c>
+      <c r="S14" s="1">
+        <v>6.2796000000000003</v>
+      </c>
+      <c r="T14" s="1">
+        <v>9.6432000000000002</v>
+      </c>
+      <c r="U14" s="1">
+        <v>51.548400000000001</v>
+      </c>
+      <c r="V14" s="28">
+        <v>1.1408E-5</v>
+      </c>
+      <c r="W14" s="1">
+        <v>21.5229</v>
+      </c>
+      <c r="X14" s="1">
+        <v>2.9426999999999999</v>
+      </c>
+      <c r="Y14" s="1">
+        <v>27.292400000000001</v>
+      </c>
+      <c r="Z14" s="1">
+        <v>20.045000000000002</v>
+      </c>
+      <c r="AA14" s="1">
+        <v>5.4419000000000004</v>
+      </c>
+      <c r="AB14" s="1">
+        <v>33.802100000000003</v>
+      </c>
+      <c r="AC14" s="1">
+        <v>47.579700000000003</v>
+      </c>
+      <c r="AD14" s="1">
+        <v>29.305399999999999</v>
+      </c>
+      <c r="AE14" s="1">
+        <v>1.3345</v>
+      </c>
+      <c r="AF14" s="1">
+        <v>21.610499999999998</v>
+      </c>
+      <c r="AG14" s="1">
+        <v>2.5678000000000001</v>
+      </c>
+      <c r="AH14" s="1">
+        <v>2.3793000000000002</v>
+      </c>
+      <c r="AI14" s="1">
+        <v>16.147300000000001</v>
+      </c>
+      <c r="AJ14" s="1">
+        <v>1.2095</v>
+      </c>
+      <c r="AK14" s="1">
+        <v>74.941500000000005</v>
+      </c>
+      <c r="AL14" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM14" s="28">
+        <v>3.0071999999999998E-4</v>
+      </c>
+      <c r="AN14" s="1">
+        <v>1.3160000000000001</v>
+      </c>
+      <c r="AO14" s="28">
+        <v>7.3287999999999999E-4</v>
+      </c>
+      <c r="AP14" s="1">
+        <v>5.0194000000000001</v>
+      </c>
+      <c r="AQ14" s="1">
+        <v>38.413699999999999</v>
+      </c>
+      <c r="AR14" s="1">
+        <v>100.9654</v>
+      </c>
+      <c r="AS14" s="1">
+        <v>1.3474999999999999</v>
+      </c>
+      <c r="AT14" s="28">
+        <v>1.3867E-15</v>
+      </c>
+      <c r="AU14" s="1">
+        <v>7.4104000000000001</v>
+      </c>
+      <c r="AV14" s="1">
+        <v>0</v>
+      </c>
+      <c r="AW14" s="1">
+        <v>2.5329999999999999</v>
+      </c>
+      <c r="AX14" s="1">
+        <v>1.4908999999999999</v>
+      </c>
+      <c r="AY14" s="1">
+        <v>11.254099999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="2:51" x14ac:dyDescent="0.3">
+      <c r="B15" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="R15" s="1">
+        <v>134.4787</v>
+      </c>
+      <c r="S15" s="1">
+        <v>2.8925000000000001</v>
+      </c>
+      <c r="T15" s="1">
+        <v>160.3175</v>
+      </c>
+      <c r="U15" s="1">
+        <v>10.509499999999999</v>
+      </c>
+      <c r="V15" s="1">
+        <v>89.633899999999997</v>
+      </c>
+      <c r="W15" s="1">
+        <v>150.1146</v>
+      </c>
+      <c r="X15" s="1">
+        <v>6.7298</v>
+      </c>
+      <c r="Y15" s="1">
+        <v>5.0404</v>
+      </c>
+      <c r="Z15" s="1">
+        <v>67.253900000000002</v>
+      </c>
+      <c r="AA15" s="28">
+        <v>1.4794999999999999E-8</v>
+      </c>
+      <c r="AB15" s="1">
+        <v>221.55369999999999</v>
+      </c>
+      <c r="AC15" s="1">
+        <v>2.8452999999999999</v>
+      </c>
+      <c r="AD15" s="1">
+        <v>2.7501000000000002</v>
+      </c>
+      <c r="AE15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AF15" s="1">
+        <v>8.4471000000000007</v>
+      </c>
+      <c r="AG15" s="1">
+        <v>1.1531</v>
+      </c>
+      <c r="AH15" s="1">
+        <v>3.3759000000000001</v>
+      </c>
+      <c r="AI15" s="1">
+        <v>1.8809</v>
+      </c>
+      <c r="AJ15" s="1">
+        <v>3.0916000000000001</v>
+      </c>
+      <c r="AK15" s="1">
+        <v>2.0199999999999999E-2</v>
+      </c>
+      <c r="AL15" s="1">
+        <v>77.834699999999998</v>
+      </c>
+      <c r="AM15" s="1">
+        <v>2.5325000000000002</v>
+      </c>
+      <c r="AN15" s="1">
+        <v>29.884899999999998</v>
+      </c>
+      <c r="AO15" s="1">
+        <v>1.8037000000000001</v>
+      </c>
+      <c r="AP15" s="1">
+        <v>0.58989999999999998</v>
+      </c>
+      <c r="AQ15" s="1">
+        <v>11.464700000000001</v>
+      </c>
+      <c r="AR15" s="1">
+        <v>6.9961000000000002</v>
+      </c>
+      <c r="AS15" s="1">
+        <v>0.56259999999999999</v>
+      </c>
+      <c r="AT15" s="1">
+        <v>13.069000000000001</v>
+      </c>
+      <c r="AU15" s="1">
+        <v>5.1165000000000003</v>
+      </c>
+      <c r="AV15" s="1">
+        <v>12.5739</v>
+      </c>
+      <c r="AW15" s="28">
+        <v>1.4433E-16</v>
+      </c>
+      <c r="AX15" s="28">
+        <v>1.6875000000000001E-16</v>
+      </c>
+      <c r="AY15" s="1">
+        <v>491.94220000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B19" s="30" t="s">
+        <v>661</v>
+      </c>
+      <c r="C19" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>663</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C3:AY15">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="10"/>
+        <cfvo type="max"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>